<commit_message>
fix: sanitizar plantilla excel eliminando table1.xml y drawing artifacts defectuosos
</commit_message>
<xml_diff>
--- a/backend/templates/2311300-FT-318_template.xlsx
+++ b/backend/templates/2311300-FT-318_template.xlsx
@@ -2260,165 +2260,7 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>1073727</xdr:colOff>
-      <xdr:row>39</xdr:row>
-      <xdr:rowOff>5773</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="101600" cy="121920"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Imagen 2">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{863EF32C-6F2D-4615-A70C-63F30D9B1467}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:srcRect/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="1521402" y="6320848"/>
-          <a:ext cx="101600" cy="121920"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>254577</xdr:colOff>
-      <xdr:row>37</xdr:row>
-      <xdr:rowOff>141143</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>454602</xdr:colOff>
-      <xdr:row>39</xdr:row>
-      <xdr:rowOff>5196</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="image3.png">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E9CF023F-7BBE-47F2-8C5A-AAB44BEC0477}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeArrowheads="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:srcRect/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="1778577" y="6132368"/>
-          <a:ext cx="200025" cy="187903"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:extLst>
-          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a14:hiddenFill>
-          </a:ext>
-          <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
-            <a14:hiddenLine xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" w="9525">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:miter lim="800000"/>
-              <a:headEnd/>
-              <a:tailEnd/>
-            </a14:hiddenLine>
-          </a:ext>
-        </a:extLst>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
 </xdr:wsDr>
-</file>
-
-<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{2FF762CF-5ECF-456A-BB17-137EEA04C074}" name="Tabla13" displayName="Tabla13" ref="A20:O31" totalsRowShown="0" headerRowDxfId="18" dataDxfId="17" headerRowBorderDxfId="15" tableBorderDxfId="16">
-  <autoFilter ref="A20:O31" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
-  <tableColumns count="15">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="ENTIDAD" dataDxfId="14"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="CARGO " dataDxfId="13"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="DESDE" dataDxfId="12"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="HASTA" dataDxfId="11"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="TIPO DE EXPERIENCIA" dataDxfId="10"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="OBSERVACIÓN" dataDxfId="9"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="FECHA EDITADA" dataDxfId="8"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="AÑOS" dataDxfId="7">
-      <calculatedColumnFormula>IF(E21="Relacionada",IF(F21="Traslape Total","-",DATEDIF(C21,D21,"Y")),"-")</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="MESES" dataDxfId="6"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="DIAS" dataDxfId="5">
-      <calculatedColumnFormula>IF(E21="Relacionada",IF(F21="Traslape Total","-",DATEDIF(C21,D21,"Md")),"-")</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="OBSERVACIÓN2" dataDxfId="4"/>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="FECHA EDITADA3" dataDxfId="3"/>
-    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="AÑOS4" dataDxfId="2">
-      <calculatedColumnFormula>IF(K21="Traslape Total","-",DATEDIF(C21,D21,"Y"))</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="MESES5" dataDxfId="1">
-      <calculatedColumnFormula>IF(K21="Traslape Total","-",DATEDIF($C21,$D21,"YM"))</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="DIAS6" dataDxfId="0">
-      <calculatedColumnFormula>IF(K21="Traslape Total","-",DATEDIF($C21,$D21,"MD"))</calculatedColumnFormula>
-    </tableColumn>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleLight8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3994,8 +3836,5 @@
   </headerFooter>
   <drawing r:id="rId3"/>
   <legacyDrawingHF r:id="rId4"/>
-  <tableParts count="1">
-    <tablePart r:id="rId5"/>
-  </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Ajustar reporte Excel: celda G8 formacion, traslape total exacto para formulas y cotejo explicito de funciones
</commit_message>
<xml_diff>
--- a/backend/templates/2311300-FT-318_template.xlsx
+++ b/backend/templates/2311300-FT-318_template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jcarl\.gemini\antigravity\scratch\administrative-requests\backend\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB7BC14D-03F3-4064-A197-2CCDA7BCA7F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C5C5547-8026-4D8A-87FD-FB00BEB2CB4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="4410" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="FORMATO" sheetId="98" r:id="rId1"/>
@@ -859,7 +859,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="118">
+  <cellXfs count="119">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -918,9 +918,6 @@
     <xf numFmtId="0" fontId="12" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -939,31 +936,68 @@
     <xf numFmtId="0" fontId="13" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="1" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -978,6 +1012,12 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="justify"/>
     </xf>
@@ -990,6 +1030,84 @@
     <xf numFmtId="15" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="6" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -1064,123 +1182,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="6" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1612,771 +1613,771 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" s="22" customFormat="1" ht="74.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="54"/>
-      <c r="B1" s="55"/>
-      <c r="C1" s="55"/>
-      <c r="D1" s="56" t="s">
+      <c r="A1" s="94"/>
+      <c r="B1" s="95"/>
+      <c r="C1" s="95"/>
+      <c r="D1" s="96" t="s">
         <v>37</v>
       </c>
-      <c r="E1" s="57"/>
-      <c r="F1" s="57"/>
-      <c r="G1" s="57"/>
-      <c r="H1" s="57"/>
-      <c r="I1" s="57"/>
-      <c r="J1" s="57"/>
-      <c r="K1" s="57"/>
-      <c r="L1" s="57"/>
-      <c r="M1" s="57"/>
-      <c r="N1" s="57"/>
-      <c r="O1" s="58"/>
+      <c r="E1" s="97"/>
+      <c r="F1" s="97"/>
+      <c r="G1" s="97"/>
+      <c r="H1" s="97"/>
+      <c r="I1" s="97"/>
+      <c r="J1" s="97"/>
+      <c r="K1" s="97"/>
+      <c r="L1" s="97"/>
+      <c r="M1" s="97"/>
+      <c r="N1" s="97"/>
+      <c r="O1" s="98"/>
     </row>
     <row r="2" spans="1:15" s="22" customFormat="1" ht="54.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="79" t="s">
+      <c r="A2" s="76" t="s">
         <v>30</v>
       </c>
-      <c r="B2" s="80"/>
-      <c r="C2" s="80"/>
-      <c r="D2" s="80"/>
-      <c r="E2" s="80"/>
-      <c r="F2" s="80"/>
-      <c r="G2" s="80"/>
-      <c r="H2" s="80"/>
-      <c r="I2" s="80"/>
-      <c r="J2" s="80"/>
-      <c r="K2" s="80"/>
-      <c r="L2" s="80"/>
-      <c r="M2" s="80"/>
-      <c r="N2" s="80"/>
-      <c r="O2" s="81"/>
+      <c r="B2" s="77"/>
+      <c r="C2" s="77"/>
+      <c r="D2" s="77"/>
+      <c r="E2" s="77"/>
+      <c r="F2" s="77"/>
+      <c r="G2" s="77"/>
+      <c r="H2" s="77"/>
+      <c r="I2" s="77"/>
+      <c r="J2" s="77"/>
+      <c r="K2" s="77"/>
+      <c r="L2" s="77"/>
+      <c r="M2" s="77"/>
+      <c r="N2" s="77"/>
+      <c r="O2" s="78"/>
     </row>
     <row r="3" spans="1:15" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="95" t="s">
+      <c r="A3" s="92" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="96"/>
-      <c r="C3" s="96"/>
-      <c r="D3" s="96"/>
-      <c r="E3" s="96"/>
-      <c r="F3" s="96"/>
-      <c r="G3" s="96"/>
-      <c r="H3" s="96"/>
-      <c r="I3" s="96"/>
-      <c r="J3" s="96"/>
-      <c r="K3" s="96"/>
-      <c r="L3" s="96"/>
-      <c r="M3" s="96"/>
-      <c r="N3" s="96"/>
+      <c r="B3" s="93"/>
+      <c r="C3" s="93"/>
+      <c r="D3" s="93"/>
+      <c r="E3" s="93"/>
+      <c r="F3" s="93"/>
+      <c r="G3" s="93"/>
+      <c r="H3" s="93"/>
+      <c r="I3" s="93"/>
+      <c r="J3" s="93"/>
+      <c r="K3" s="93"/>
+      <c r="L3" s="93"/>
+      <c r="M3" s="93"/>
+      <c r="N3" s="93"/>
       <c r="O3" s="13"/>
     </row>
     <row r="4" spans="1:15" ht="32.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="15" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="69"/>
-      <c r="C4" s="69"/>
-      <c r="D4" s="91" t="s">
+      <c r="B4" s="109"/>
+      <c r="C4" s="109"/>
+      <c r="D4" s="88" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="91"/>
-      <c r="F4" s="74"/>
-      <c r="G4" s="75"/>
+      <c r="E4" s="88"/>
+      <c r="F4" s="114"/>
+      <c r="G4" s="115"/>
       <c r="H4" s="16" t="s">
         <v>28</v>
       </c>
-      <c r="I4" s="70"/>
-      <c r="J4" s="71"/>
-      <c r="K4" s="69" t="s">
+      <c r="I4" s="110"/>
+      <c r="J4" s="111"/>
+      <c r="K4" s="109" t="s">
         <v>29</v>
       </c>
-      <c r="L4" s="69"/>
-      <c r="M4" s="76"/>
-      <c r="N4" s="77"/>
-      <c r="O4" s="78"/>
+      <c r="L4" s="109"/>
+      <c r="M4" s="116"/>
+      <c r="N4" s="117"/>
+      <c r="O4" s="118"/>
     </row>
     <row r="5" spans="1:15" ht="32.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A5" s="17" t="s">
         <v>47</v>
       </c>
-      <c r="B5" s="48"/>
-      <c r="C5" s="48"/>
+      <c r="B5" s="60"/>
+      <c r="C5" s="60"/>
       <c r="D5" s="18" t="s">
         <v>7</v>
       </c>
-      <c r="E5" s="92"/>
-      <c r="F5" s="93"/>
-      <c r="G5" s="94"/>
-      <c r="H5" s="47" t="s">
+      <c r="E5" s="89"/>
+      <c r="F5" s="90"/>
+      <c r="G5" s="91"/>
+      <c r="H5" s="59" t="s">
         <v>10</v>
       </c>
-      <c r="I5" s="47"/>
-      <c r="J5" s="48"/>
-      <c r="K5" s="48"/>
-      <c r="L5" s="47" t="s">
+      <c r="I5" s="59"/>
+      <c r="J5" s="60"/>
+      <c r="K5" s="60"/>
+      <c r="L5" s="59" t="s">
         <v>11</v>
       </c>
-      <c r="M5" s="47"/>
-      <c r="N5" s="72"/>
-      <c r="O5" s="73"/>
+      <c r="M5" s="59"/>
+      <c r="N5" s="112"/>
+      <c r="O5" s="113"/>
     </row>
     <row r="6" spans="1:15" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="82" t="s">
+      <c r="A6" s="79" t="s">
         <v>15</v>
       </c>
-      <c r="B6" s="83"/>
-      <c r="C6" s="83"/>
-      <c r="D6" s="83"/>
-      <c r="E6" s="83"/>
-      <c r="F6" s="83"/>
-      <c r="G6" s="83"/>
-      <c r="H6" s="83"/>
-      <c r="I6" s="83"/>
-      <c r="J6" s="83"/>
-      <c r="K6" s="83"/>
-      <c r="L6" s="83"/>
-      <c r="M6" s="83"/>
-      <c r="N6" s="83"/>
-      <c r="O6" s="84"/>
+      <c r="B6" s="80"/>
+      <c r="C6" s="80"/>
+      <c r="D6" s="80"/>
+      <c r="E6" s="80"/>
+      <c r="F6" s="80"/>
+      <c r="G6" s="80"/>
+      <c r="H6" s="80"/>
+      <c r="I6" s="80"/>
+      <c r="J6" s="80"/>
+      <c r="K6" s="80"/>
+      <c r="L6" s="80"/>
+      <c r="M6" s="80"/>
+      <c r="N6" s="80"/>
+      <c r="O6" s="81"/>
     </row>
     <row r="7" spans="1:15" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="64" t="s">
+      <c r="A7" s="104" t="s">
         <v>14</v>
       </c>
-      <c r="B7" s="65"/>
-      <c r="C7" s="65"/>
-      <c r="D7" s="65"/>
-      <c r="E7" s="65"/>
-      <c r="F7" s="66"/>
-      <c r="G7" s="67" t="s">
+      <c r="B7" s="105"/>
+      <c r="C7" s="105"/>
+      <c r="D7" s="105"/>
+      <c r="E7" s="105"/>
+      <c r="F7" s="106"/>
+      <c r="G7" s="107" t="s">
         <v>13</v>
       </c>
-      <c r="H7" s="65"/>
-      <c r="I7" s="65"/>
-      <c r="J7" s="65"/>
-      <c r="K7" s="65"/>
-      <c r="L7" s="65"/>
-      <c r="M7" s="65"/>
-      <c r="N7" s="65"/>
-      <c r="O7" s="68"/>
+      <c r="H7" s="105"/>
+      <c r="I7" s="105"/>
+      <c r="J7" s="105"/>
+      <c r="K7" s="105"/>
+      <c r="L7" s="105"/>
+      <c r="M7" s="105"/>
+      <c r="N7" s="105"/>
+      <c r="O7" s="108"/>
     </row>
     <row r="8" spans="1:15" ht="148.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="59"/>
-      <c r="B8" s="60"/>
-      <c r="C8" s="60"/>
-      <c r="D8" s="60"/>
-      <c r="E8" s="60"/>
-      <c r="F8" s="60"/>
-      <c r="G8" s="61"/>
-      <c r="H8" s="62"/>
-      <c r="I8" s="62"/>
-      <c r="J8" s="62"/>
-      <c r="K8" s="62"/>
-      <c r="L8" s="62"/>
-      <c r="M8" s="62"/>
-      <c r="N8" s="62"/>
-      <c r="O8" s="63"/>
+      <c r="A8" s="99"/>
+      <c r="B8" s="100"/>
+      <c r="C8" s="100"/>
+      <c r="D8" s="100"/>
+      <c r="E8" s="100"/>
+      <c r="F8" s="100"/>
+      <c r="G8" s="101"/>
+      <c r="H8" s="102"/>
+      <c r="I8" s="102"/>
+      <c r="J8" s="102"/>
+      <c r="K8" s="102"/>
+      <c r="L8" s="102"/>
+      <c r="M8" s="102"/>
+      <c r="N8" s="102"/>
+      <c r="O8" s="103"/>
     </row>
     <row r="9" spans="1:15" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="85" t="s">
+      <c r="A9" s="82" t="s">
         <v>16</v>
       </c>
-      <c r="B9" s="86"/>
-      <c r="C9" s="86"/>
-      <c r="D9" s="86"/>
-      <c r="E9" s="86"/>
-      <c r="F9" s="86"/>
-      <c r="G9" s="86"/>
-      <c r="H9" s="86"/>
-      <c r="I9" s="86"/>
-      <c r="J9" s="86"/>
-      <c r="K9" s="86"/>
-      <c r="L9" s="86"/>
-      <c r="M9" s="86"/>
-      <c r="N9" s="86"/>
-      <c r="O9" s="87"/>
+      <c r="B9" s="83"/>
+      <c r="C9" s="83"/>
+      <c r="D9" s="83"/>
+      <c r="E9" s="83"/>
+      <c r="F9" s="83"/>
+      <c r="G9" s="83"/>
+      <c r="H9" s="83"/>
+      <c r="I9" s="83"/>
+      <c r="J9" s="83"/>
+      <c r="K9" s="83"/>
+      <c r="L9" s="83"/>
+      <c r="M9" s="83"/>
+      <c r="N9" s="83"/>
+      <c r="O9" s="84"/>
     </row>
     <row r="10" spans="1:15" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="88" t="s">
+      <c r="A10" s="85" t="s">
         <v>18</v>
       </c>
-      <c r="B10" s="89"/>
-      <c r="C10" s="89"/>
-      <c r="D10" s="89"/>
-      <c r="E10" s="89"/>
-      <c r="F10" s="89"/>
-      <c r="G10" s="89"/>
-      <c r="H10" s="89"/>
-      <c r="I10" s="89"/>
-      <c r="J10" s="89"/>
-      <c r="K10" s="89"/>
-      <c r="L10" s="89"/>
-      <c r="M10" s="89"/>
-      <c r="N10" s="89"/>
-      <c r="O10" s="90"/>
+      <c r="B10" s="86"/>
+      <c r="C10" s="86"/>
+      <c r="D10" s="86"/>
+      <c r="E10" s="86"/>
+      <c r="F10" s="86"/>
+      <c r="G10" s="86"/>
+      <c r="H10" s="86"/>
+      <c r="I10" s="86"/>
+      <c r="J10" s="86"/>
+      <c r="K10" s="86"/>
+      <c r="L10" s="86"/>
+      <c r="M10" s="86"/>
+      <c r="N10" s="86"/>
+      <c r="O10" s="87"/>
     </row>
     <row r="11" spans="1:15" ht="34.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="108" t="s">
+      <c r="A11" s="36" t="s">
         <v>39</v>
       </c>
-      <c r="B11" s="109"/>
-      <c r="C11" s="109"/>
-      <c r="D11" s="109"/>
-      <c r="E11" s="110" t="s">
+      <c r="B11" s="62"/>
+      <c r="C11" s="62"/>
+      <c r="D11" s="62"/>
+      <c r="E11" s="47" t="s">
         <v>25</v>
       </c>
-      <c r="F11" s="110"/>
-      <c r="G11" s="110"/>
-      <c r="H11" s="109"/>
-      <c r="I11" s="109"/>
-      <c r="J11" s="109"/>
-      <c r="K11" s="109"/>
-      <c r="L11" s="110" t="s">
+      <c r="F11" s="47"/>
+      <c r="G11" s="47"/>
+      <c r="H11" s="62"/>
+      <c r="I11" s="62"/>
+      <c r="J11" s="62"/>
+      <c r="K11" s="62"/>
+      <c r="L11" s="47" t="s">
         <v>26</v>
       </c>
-      <c r="M11" s="110"/>
-      <c r="N11" s="111"/>
-      <c r="O11" s="112"/>
+      <c r="M11" s="47"/>
+      <c r="N11" s="70"/>
+      <c r="O11" s="71"/>
     </row>
     <row r="12" spans="1:15" ht="34.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="B12" s="99"/>
-      <c r="C12" s="100"/>
-      <c r="D12" s="101"/>
-      <c r="E12" s="97" t="s">
+      <c r="B12" s="42"/>
+      <c r="C12" s="43"/>
+      <c r="D12" s="44"/>
+      <c r="E12" s="55" t="s">
         <v>25</v>
       </c>
-      <c r="F12" s="102"/>
-      <c r="G12" s="98"/>
-      <c r="H12" s="99"/>
-      <c r="I12" s="100"/>
-      <c r="J12" s="100"/>
-      <c r="K12" s="101"/>
-      <c r="L12" s="97" t="s">
+      <c r="F12" s="56"/>
+      <c r="G12" s="57"/>
+      <c r="H12" s="42"/>
+      <c r="I12" s="43"/>
+      <c r="J12" s="43"/>
+      <c r="K12" s="44"/>
+      <c r="L12" s="55" t="s">
         <v>26</v>
       </c>
-      <c r="M12" s="98"/>
-      <c r="N12" s="103"/>
-      <c r="O12" s="104"/>
+      <c r="M12" s="57"/>
+      <c r="N12" s="68"/>
+      <c r="O12" s="69"/>
     </row>
     <row r="13" spans="1:15" ht="34.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="B13" s="99"/>
-      <c r="C13" s="100"/>
-      <c r="D13" s="101"/>
-      <c r="E13" s="97" t="s">
+      <c r="B13" s="42"/>
+      <c r="C13" s="43"/>
+      <c r="D13" s="44"/>
+      <c r="E13" s="55" t="s">
         <v>25</v>
       </c>
-      <c r="F13" s="102"/>
-      <c r="G13" s="98"/>
-      <c r="H13" s="99"/>
-      <c r="I13" s="100"/>
-      <c r="J13" s="100"/>
-      <c r="K13" s="101"/>
-      <c r="L13" s="97" t="s">
+      <c r="F13" s="56"/>
+      <c r="G13" s="57"/>
+      <c r="H13" s="42"/>
+      <c r="I13" s="43"/>
+      <c r="J13" s="43"/>
+      <c r="K13" s="44"/>
+      <c r="L13" s="55" t="s">
         <v>26</v>
       </c>
-      <c r="M13" s="98"/>
-      <c r="N13" s="103"/>
-      <c r="O13" s="104"/>
+      <c r="M13" s="57"/>
+      <c r="N13" s="68"/>
+      <c r="O13" s="69"/>
     </row>
     <row r="14" spans="1:15" ht="34.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="B14" s="99"/>
-      <c r="C14" s="100"/>
-      <c r="D14" s="101"/>
-      <c r="E14" s="97" t="s">
+      <c r="B14" s="42"/>
+      <c r="C14" s="43"/>
+      <c r="D14" s="44"/>
+      <c r="E14" s="55" t="s">
         <v>25</v>
       </c>
-      <c r="F14" s="102"/>
-      <c r="G14" s="98"/>
-      <c r="H14" s="99"/>
-      <c r="I14" s="100"/>
-      <c r="J14" s="100"/>
-      <c r="K14" s="101"/>
-      <c r="L14" s="97" t="s">
+      <c r="F14" s="56"/>
+      <c r="G14" s="57"/>
+      <c r="H14" s="42"/>
+      <c r="I14" s="43"/>
+      <c r="J14" s="43"/>
+      <c r="K14" s="44"/>
+      <c r="L14" s="55" t="s">
         <v>26</v>
       </c>
-      <c r="M14" s="98"/>
-      <c r="N14" s="103"/>
-      <c r="O14" s="104"/>
+      <c r="M14" s="57"/>
+      <c r="N14" s="68"/>
+      <c r="O14" s="69"/>
     </row>
     <row r="15" spans="1:15" ht="34.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="B15" s="99"/>
-      <c r="C15" s="100"/>
-      <c r="D15" s="101"/>
-      <c r="E15" s="97" t="s">
+      <c r="B15" s="42"/>
+      <c r="C15" s="43"/>
+      <c r="D15" s="44"/>
+      <c r="E15" s="55" t="s">
         <v>25</v>
       </c>
-      <c r="F15" s="102"/>
-      <c r="G15" s="98"/>
-      <c r="H15" s="99"/>
-      <c r="I15" s="100"/>
-      <c r="J15" s="100"/>
-      <c r="K15" s="101"/>
-      <c r="L15" s="97" t="s">
+      <c r="F15" s="56"/>
+      <c r="G15" s="57"/>
+      <c r="H15" s="42"/>
+      <c r="I15" s="43"/>
+      <c r="J15" s="43"/>
+      <c r="K15" s="44"/>
+      <c r="L15" s="55" t="s">
         <v>26</v>
       </c>
-      <c r="M15" s="98"/>
-      <c r="N15" s="103"/>
-      <c r="O15" s="104"/>
+      <c r="M15" s="57"/>
+      <c r="N15" s="68"/>
+      <c r="O15" s="69"/>
     </row>
     <row r="16" spans="1:15" ht="34.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="12" t="s">
         <v>50</v>
       </c>
-      <c r="B16" s="99"/>
-      <c r="C16" s="100"/>
-      <c r="D16" s="101"/>
-      <c r="E16" s="97" t="s">
+      <c r="B16" s="42"/>
+      <c r="C16" s="43"/>
+      <c r="D16" s="44"/>
+      <c r="E16" s="55" t="s">
         <v>25</v>
       </c>
-      <c r="F16" s="102"/>
-      <c r="G16" s="98"/>
-      <c r="H16" s="99"/>
-      <c r="I16" s="100"/>
-      <c r="J16" s="100"/>
-      <c r="K16" s="101"/>
-      <c r="L16" s="97" t="s">
+      <c r="F16" s="56"/>
+      <c r="G16" s="57"/>
+      <c r="H16" s="42"/>
+      <c r="I16" s="43"/>
+      <c r="J16" s="43"/>
+      <c r="K16" s="44"/>
+      <c r="L16" s="55" t="s">
         <v>26</v>
       </c>
-      <c r="M16" s="98"/>
-      <c r="N16" s="103"/>
-      <c r="O16" s="104"/>
+      <c r="M16" s="57"/>
+      <c r="N16" s="68"/>
+      <c r="O16" s="69"/>
     </row>
     <row r="17" spans="1:15" ht="34.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="12" t="s">
         <v>50</v>
       </c>
-      <c r="B17" s="99"/>
-      <c r="C17" s="100"/>
-      <c r="D17" s="101"/>
-      <c r="E17" s="97" t="s">
+      <c r="B17" s="42"/>
+      <c r="C17" s="43"/>
+      <c r="D17" s="44"/>
+      <c r="E17" s="55" t="s">
         <v>25</v>
       </c>
-      <c r="F17" s="102"/>
-      <c r="G17" s="98"/>
-      <c r="H17" s="99"/>
-      <c r="I17" s="100"/>
-      <c r="J17" s="100"/>
-      <c r="K17" s="101"/>
-      <c r="L17" s="97" t="s">
+      <c r="F17" s="56"/>
+      <c r="G17" s="57"/>
+      <c r="H17" s="42"/>
+      <c r="I17" s="43"/>
+      <c r="J17" s="43"/>
+      <c r="K17" s="44"/>
+      <c r="L17" s="55" t="s">
         <v>26</v>
       </c>
-      <c r="M17" s="98"/>
-      <c r="N17" s="103"/>
-      <c r="O17" s="104"/>
+      <c r="M17" s="57"/>
+      <c r="N17" s="68"/>
+      <c r="O17" s="69"/>
     </row>
     <row r="18" spans="1:15" ht="34.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="12" t="s">
         <v>50</v>
       </c>
-      <c r="B18" s="99"/>
-      <c r="C18" s="100"/>
-      <c r="D18" s="101"/>
-      <c r="E18" s="97" t="s">
+      <c r="B18" s="42"/>
+      <c r="C18" s="43"/>
+      <c r="D18" s="44"/>
+      <c r="E18" s="55" t="s">
         <v>25</v>
       </c>
-      <c r="F18" s="102"/>
-      <c r="G18" s="98"/>
-      <c r="H18" s="99"/>
-      <c r="I18" s="100"/>
-      <c r="J18" s="100"/>
-      <c r="K18" s="101"/>
-      <c r="L18" s="97" t="s">
+      <c r="F18" s="56"/>
+      <c r="G18" s="57"/>
+      <c r="H18" s="42"/>
+      <c r="I18" s="43"/>
+      <c r="J18" s="43"/>
+      <c r="K18" s="44"/>
+      <c r="L18" s="55" t="s">
         <v>26</v>
       </c>
-      <c r="M18" s="98"/>
-      <c r="N18" s="103"/>
-      <c r="O18" s="104"/>
+      <c r="M18" s="57"/>
+      <c r="N18" s="68"/>
+      <c r="O18" s="69"/>
     </row>
     <row r="19" spans="1:15" ht="34.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="12" t="s">
         <v>50</v>
       </c>
-      <c r="B19" s="99"/>
-      <c r="C19" s="100"/>
-      <c r="D19" s="101"/>
-      <c r="E19" s="97" t="s">
+      <c r="B19" s="42"/>
+      <c r="C19" s="43"/>
+      <c r="D19" s="44"/>
+      <c r="E19" s="55" t="s">
         <v>25</v>
       </c>
-      <c r="F19" s="102"/>
-      <c r="G19" s="98"/>
-      <c r="H19" s="99"/>
-      <c r="I19" s="100"/>
-      <c r="J19" s="100"/>
-      <c r="K19" s="101"/>
-      <c r="L19" s="97" t="s">
+      <c r="F19" s="56"/>
+      <c r="G19" s="57"/>
+      <c r="H19" s="42"/>
+      <c r="I19" s="43"/>
+      <c r="J19" s="43"/>
+      <c r="K19" s="44"/>
+      <c r="L19" s="55" t="s">
         <v>26</v>
       </c>
-      <c r="M19" s="98"/>
-      <c r="N19" s="103"/>
-      <c r="O19" s="104"/>
+      <c r="M19" s="57"/>
+      <c r="N19" s="68"/>
+      <c r="O19" s="69"/>
     </row>
     <row r="20" spans="1:15" ht="34.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="B20" s="43"/>
-      <c r="C20" s="43"/>
-      <c r="D20" s="43"/>
-      <c r="E20" s="45" t="s">
+      <c r="B20" s="51"/>
+      <c r="C20" s="51"/>
+      <c r="D20" s="51"/>
+      <c r="E20" s="63" t="s">
         <v>25</v>
       </c>
-      <c r="F20" s="45"/>
-      <c r="G20" s="45"/>
-      <c r="H20" s="42"/>
-      <c r="I20" s="42"/>
-      <c r="J20" s="42"/>
-      <c r="K20" s="42"/>
-      <c r="L20" s="45" t="s">
+      <c r="F20" s="63"/>
+      <c r="G20" s="63"/>
+      <c r="H20" s="52"/>
+      <c r="I20" s="52"/>
+      <c r="J20" s="52"/>
+      <c r="K20" s="52"/>
+      <c r="L20" s="63" t="s">
         <v>26</v>
       </c>
-      <c r="M20" s="45"/>
-      <c r="N20" s="37"/>
-      <c r="O20" s="38"/>
+      <c r="M20" s="63"/>
+      <c r="N20" s="49"/>
+      <c r="O20" s="50"/>
     </row>
     <row r="21" spans="1:15" ht="34.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="B21" s="43"/>
-      <c r="C21" s="43"/>
-      <c r="D21" s="43"/>
-      <c r="E21" s="45" t="s">
+      <c r="B21" s="51"/>
+      <c r="C21" s="51"/>
+      <c r="D21" s="51"/>
+      <c r="E21" s="63" t="s">
         <v>25</v>
       </c>
-      <c r="F21" s="45"/>
-      <c r="G21" s="45"/>
-      <c r="H21" s="42"/>
-      <c r="I21" s="42"/>
-      <c r="J21" s="42"/>
-      <c r="K21" s="42"/>
-      <c r="L21" s="45" t="s">
+      <c r="F21" s="63"/>
+      <c r="G21" s="63"/>
+      <c r="H21" s="52"/>
+      <c r="I21" s="52"/>
+      <c r="J21" s="52"/>
+      <c r="K21" s="52"/>
+      <c r="L21" s="63" t="s">
         <v>26</v>
       </c>
-      <c r="M21" s="45"/>
-      <c r="N21" s="37"/>
-      <c r="O21" s="38"/>
+      <c r="M21" s="63"/>
+      <c r="N21" s="49"/>
+      <c r="O21" s="50"/>
     </row>
     <row r="22" spans="1:15" ht="34.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="B22" s="43"/>
-      <c r="C22" s="43"/>
-      <c r="D22" s="43"/>
-      <c r="E22" s="45" t="s">
+      <c r="B22" s="51"/>
+      <c r="C22" s="51"/>
+      <c r="D22" s="51"/>
+      <c r="E22" s="63" t="s">
         <v>25</v>
       </c>
-      <c r="F22" s="45"/>
-      <c r="G22" s="45"/>
-      <c r="H22" s="42"/>
-      <c r="I22" s="42"/>
-      <c r="J22" s="42"/>
-      <c r="K22" s="42"/>
-      <c r="L22" s="45" t="s">
+      <c r="F22" s="63"/>
+      <c r="G22" s="63"/>
+      <c r="H22" s="52"/>
+      <c r="I22" s="52"/>
+      <c r="J22" s="52"/>
+      <c r="K22" s="52"/>
+      <c r="L22" s="63" t="s">
         <v>26</v>
       </c>
-      <c r="M22" s="45"/>
-      <c r="N22" s="37"/>
-      <c r="O22" s="38"/>
+      <c r="M22" s="63"/>
+      <c r="N22" s="49"/>
+      <c r="O22" s="50"/>
     </row>
     <row r="23" spans="1:15" ht="34.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="B23" s="43"/>
-      <c r="C23" s="43"/>
-      <c r="D23" s="43"/>
-      <c r="E23" s="45" t="s">
+      <c r="B23" s="51"/>
+      <c r="C23" s="51"/>
+      <c r="D23" s="51"/>
+      <c r="E23" s="63" t="s">
         <v>25</v>
       </c>
-      <c r="F23" s="45"/>
-      <c r="G23" s="45"/>
-      <c r="H23" s="42"/>
-      <c r="I23" s="42"/>
-      <c r="J23" s="42"/>
-      <c r="K23" s="42"/>
-      <c r="L23" s="45" t="s">
+      <c r="F23" s="63"/>
+      <c r="G23" s="63"/>
+      <c r="H23" s="52"/>
+      <c r="I23" s="52"/>
+      <c r="J23" s="52"/>
+      <c r="K23" s="52"/>
+      <c r="L23" s="63" t="s">
         <v>26</v>
       </c>
-      <c r="M23" s="45"/>
-      <c r="N23" s="37"/>
-      <c r="O23" s="38"/>
+      <c r="M23" s="63"/>
+      <c r="N23" s="49"/>
+      <c r="O23" s="50"/>
     </row>
     <row r="24" spans="1:15" ht="34.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="B24" s="44"/>
-      <c r="C24" s="44"/>
-      <c r="D24" s="44"/>
-      <c r="E24" s="41" t="s">
+      <c r="B24" s="46"/>
+      <c r="C24" s="46"/>
+      <c r="D24" s="46"/>
+      <c r="E24" s="45" t="s">
         <v>25</v>
       </c>
-      <c r="F24" s="41"/>
-      <c r="G24" s="41"/>
-      <c r="H24" s="42"/>
-      <c r="I24" s="42"/>
-      <c r="J24" s="42"/>
-      <c r="K24" s="42"/>
-      <c r="L24" s="41" t="s">
+      <c r="F24" s="45"/>
+      <c r="G24" s="45"/>
+      <c r="H24" s="52"/>
+      <c r="I24" s="52"/>
+      <c r="J24" s="52"/>
+      <c r="K24" s="52"/>
+      <c r="L24" s="45" t="s">
         <v>26</v>
       </c>
-      <c r="M24" s="41"/>
-      <c r="N24" s="39"/>
-      <c r="O24" s="40"/>
+      <c r="M24" s="45"/>
+      <c r="N24" s="53"/>
+      <c r="O24" s="54"/>
     </row>
     <row r="25" spans="1:15" ht="34.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="B25" s="44"/>
-      <c r="C25" s="44"/>
-      <c r="D25" s="44"/>
-      <c r="E25" s="41" t="s">
+      <c r="B25" s="46"/>
+      <c r="C25" s="46"/>
+      <c r="D25" s="46"/>
+      <c r="E25" s="45" t="s">
         <v>25</v>
       </c>
-      <c r="F25" s="41"/>
-      <c r="G25" s="41"/>
-      <c r="H25" s="42"/>
-      <c r="I25" s="42"/>
-      <c r="J25" s="42"/>
-      <c r="K25" s="42"/>
-      <c r="L25" s="41" t="s">
+      <c r="F25" s="45"/>
+      <c r="G25" s="45"/>
+      <c r="H25" s="52"/>
+      <c r="I25" s="52"/>
+      <c r="J25" s="52"/>
+      <c r="K25" s="52"/>
+      <c r="L25" s="45" t="s">
         <v>26</v>
       </c>
-      <c r="M25" s="41"/>
-      <c r="N25" s="39"/>
-      <c r="O25" s="40"/>
+      <c r="M25" s="45"/>
+      <c r="N25" s="53"/>
+      <c r="O25" s="54"/>
     </row>
     <row r="26" spans="1:15" ht="34.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="B26" s="44"/>
-      <c r="C26" s="44"/>
-      <c r="D26" s="44"/>
-      <c r="E26" s="41" t="s">
+      <c r="B26" s="46"/>
+      <c r="C26" s="46"/>
+      <c r="D26" s="46"/>
+      <c r="E26" s="45" t="s">
         <v>25</v>
       </c>
-      <c r="F26" s="41"/>
-      <c r="G26" s="41"/>
-      <c r="H26" s="42"/>
-      <c r="I26" s="42"/>
-      <c r="J26" s="42"/>
-      <c r="K26" s="42"/>
-      <c r="L26" s="41" t="s">
+      <c r="F26" s="45"/>
+      <c r="G26" s="45"/>
+      <c r="H26" s="52"/>
+      <c r="I26" s="52"/>
+      <c r="J26" s="52"/>
+      <c r="K26" s="52"/>
+      <c r="L26" s="45" t="s">
         <v>26</v>
       </c>
-      <c r="M26" s="41"/>
-      <c r="N26" s="39"/>
-      <c r="O26" s="40"/>
+      <c r="M26" s="45"/>
+      <c r="N26" s="53"/>
+      <c r="O26" s="54"/>
     </row>
     <row r="27" spans="1:15" ht="34.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="B27" s="44"/>
-      <c r="C27" s="44"/>
-      <c r="D27" s="44"/>
-      <c r="E27" s="41" t="s">
+      <c r="B27" s="46"/>
+      <c r="C27" s="46"/>
+      <c r="D27" s="46"/>
+      <c r="E27" s="45" t="s">
         <v>25</v>
       </c>
-      <c r="F27" s="41"/>
-      <c r="G27" s="41"/>
-      <c r="H27" s="42"/>
-      <c r="I27" s="42"/>
-      <c r="J27" s="42"/>
-      <c r="K27" s="42"/>
-      <c r="L27" s="41" t="s">
+      <c r="F27" s="45"/>
+      <c r="G27" s="45"/>
+      <c r="H27" s="52"/>
+      <c r="I27" s="52"/>
+      <c r="J27" s="52"/>
+      <c r="K27" s="52"/>
+      <c r="L27" s="45" t="s">
         <v>26</v>
       </c>
-      <c r="M27" s="41"/>
-      <c r="N27" s="39"/>
-      <c r="O27" s="40"/>
+      <c r="M27" s="45"/>
+      <c r="N27" s="53"/>
+      <c r="O27" s="54"/>
     </row>
     <row r="28" spans="1:15" ht="34.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="B28" s="44"/>
-      <c r="C28" s="44"/>
-      <c r="D28" s="44"/>
-      <c r="E28" s="41" t="s">
+      <c r="B28" s="46"/>
+      <c r="C28" s="46"/>
+      <c r="D28" s="46"/>
+      <c r="E28" s="45" t="s">
         <v>25</v>
       </c>
-      <c r="F28" s="41"/>
-      <c r="G28" s="41"/>
-      <c r="H28" s="42"/>
-      <c r="I28" s="42"/>
-      <c r="J28" s="42"/>
-      <c r="K28" s="42"/>
-      <c r="L28" s="41" t="s">
+      <c r="F28" s="45"/>
+      <c r="G28" s="45"/>
+      <c r="H28" s="52"/>
+      <c r="I28" s="52"/>
+      <c r="J28" s="52"/>
+      <c r="K28" s="52"/>
+      <c r="L28" s="45" t="s">
         <v>26</v>
       </c>
-      <c r="M28" s="41"/>
-      <c r="N28" s="39"/>
-      <c r="O28" s="40"/>
+      <c r="M28" s="45"/>
+      <c r="N28" s="53"/>
+      <c r="O28" s="54"/>
     </row>
     <row r="29" spans="1:15" ht="34.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="B29" s="44"/>
-      <c r="C29" s="44"/>
-      <c r="D29" s="44"/>
-      <c r="E29" s="41" t="s">
+      <c r="B29" s="46"/>
+      <c r="C29" s="46"/>
+      <c r="D29" s="46"/>
+      <c r="E29" s="45" t="s">
         <v>25</v>
       </c>
-      <c r="F29" s="41"/>
-      <c r="G29" s="41"/>
-      <c r="H29" s="42"/>
-      <c r="I29" s="42"/>
-      <c r="J29" s="42"/>
-      <c r="K29" s="42"/>
-      <c r="L29" s="41" t="s">
+      <c r="F29" s="45"/>
+      <c r="G29" s="45"/>
+      <c r="H29" s="52"/>
+      <c r="I29" s="52"/>
+      <c r="J29" s="52"/>
+      <c r="K29" s="52"/>
+      <c r="L29" s="45" t="s">
         <v>26</v>
       </c>
-      <c r="M29" s="41"/>
-      <c r="N29" s="39"/>
-      <c r="O29" s="40"/>
+      <c r="M29" s="45"/>
+      <c r="N29" s="53"/>
+      <c r="O29" s="54"/>
     </row>
     <row r="30" spans="1:15" ht="34.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="B30" s="44"/>
-      <c r="C30" s="44"/>
-      <c r="D30" s="44"/>
-      <c r="E30" s="41" t="s">
+      <c r="B30" s="46"/>
+      <c r="C30" s="46"/>
+      <c r="D30" s="46"/>
+      <c r="E30" s="45" t="s">
         <v>25</v>
       </c>
-      <c r="F30" s="41"/>
-      <c r="G30" s="41"/>
-      <c r="H30" s="42"/>
-      <c r="I30" s="42"/>
-      <c r="J30" s="42"/>
-      <c r="K30" s="42"/>
-      <c r="L30" s="41" t="s">
+      <c r="F30" s="45"/>
+      <c r="G30" s="45"/>
+      <c r="H30" s="52"/>
+      <c r="I30" s="52"/>
+      <c r="J30" s="52"/>
+      <c r="K30" s="52"/>
+      <c r="L30" s="45" t="s">
         <v>26</v>
       </c>
-      <c r="M30" s="41"/>
-      <c r="N30" s="39"/>
-      <c r="O30" s="40"/>
+      <c r="M30" s="45"/>
+      <c r="N30" s="53"/>
+      <c r="O30" s="54"/>
     </row>
     <row r="31" spans="1:15" ht="34.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="B31" s="44"/>
-      <c r="C31" s="44"/>
-      <c r="D31" s="44"/>
-      <c r="E31" s="41" t="s">
+      <c r="B31" s="46"/>
+      <c r="C31" s="46"/>
+      <c r="D31" s="46"/>
+      <c r="E31" s="45" t="s">
         <v>25</v>
       </c>
-      <c r="F31" s="41"/>
-      <c r="G31" s="41"/>
-      <c r="H31" s="42"/>
-      <c r="I31" s="42"/>
-      <c r="J31" s="42"/>
-      <c r="K31" s="42"/>
-      <c r="L31" s="41" t="s">
+      <c r="F31" s="45"/>
+      <c r="G31" s="45"/>
+      <c r="H31" s="52"/>
+      <c r="I31" s="52"/>
+      <c r="J31" s="52"/>
+      <c r="K31" s="52"/>
+      <c r="L31" s="45" t="s">
         <v>26</v>
       </c>
-      <c r="M31" s="41"/>
-      <c r="N31" s="39"/>
-      <c r="O31" s="40"/>
+      <c r="M31" s="45"/>
+      <c r="N31" s="53"/>
+      <c r="O31" s="54"/>
     </row>
     <row r="32" spans="1:15" ht="34.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="113" t="s">
+      <c r="A32" s="37" t="s">
         <v>9</v>
       </c>
-      <c r="B32" s="114"/>
-      <c r="C32" s="114"/>
-      <c r="D32" s="114"/>
-      <c r="E32" s="115" t="s">
+      <c r="B32" s="48"/>
+      <c r="C32" s="48"/>
+      <c r="D32" s="48"/>
+      <c r="E32" s="75" t="s">
         <v>27</v>
       </c>
-      <c r="F32" s="115"/>
-      <c r="G32" s="115"/>
-      <c r="H32" s="114"/>
-      <c r="I32" s="114"/>
-      <c r="J32" s="114"/>
-      <c r="K32" s="114"/>
-      <c r="L32" s="116"/>
-      <c r="M32" s="116"/>
-      <c r="N32" s="116"/>
-      <c r="O32" s="117"/>
+      <c r="F32" s="75"/>
+      <c r="G32" s="75"/>
+      <c r="H32" s="48"/>
+      <c r="I32" s="48"/>
+      <c r="J32" s="48"/>
+      <c r="K32" s="48"/>
+      <c r="L32" s="38"/>
+      <c r="M32" s="38"/>
+      <c r="N32" s="38"/>
+      <c r="O32" s="39"/>
     </row>
     <row r="33" spans="1:15" ht="27" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="106" t="s">
+      <c r="A33" s="72" t="s">
         <v>17</v>
       </c>
-      <c r="B33" s="105"/>
-      <c r="C33" s="105"/>
-      <c r="D33" s="105"/>
-      <c r="E33" s="105"/>
-      <c r="F33" s="105"/>
-      <c r="G33" s="105"/>
-      <c r="H33" s="105"/>
-      <c r="I33" s="105"/>
-      <c r="J33" s="105"/>
-      <c r="K33" s="105"/>
-      <c r="L33" s="105"/>
-      <c r="M33" s="105"/>
-      <c r="N33" s="105"/>
-      <c r="O33" s="107"/>
+      <c r="B33" s="73"/>
+      <c r="C33" s="73"/>
+      <c r="D33" s="73"/>
+      <c r="E33" s="73"/>
+      <c r="F33" s="73"/>
+      <c r="G33" s="73"/>
+      <c r="H33" s="73"/>
+      <c r="I33" s="73"/>
+      <c r="J33" s="73"/>
+      <c r="K33" s="73"/>
+      <c r="L33" s="73"/>
+      <c r="M33" s="73"/>
+      <c r="N33" s="73"/>
+      <c r="O33" s="74"/>
     </row>
     <row r="34" spans="1:15" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="52" t="s">
+      <c r="A34" s="66" t="s">
         <v>23</v>
       </c>
-      <c r="B34" s="52" t="s">
+      <c r="B34" s="66" t="s">
         <v>24</v>
       </c>
-      <c r="C34" s="53" t="s">
+      <c r="C34" s="67" t="s">
         <v>19</v>
       </c>
-      <c r="D34" s="53" t="s">
+      <c r="D34" s="67" t="s">
         <v>20</v>
       </c>
-      <c r="E34" s="53" t="s">
+      <c r="E34" s="67" t="s">
         <v>12</v>
       </c>
-      <c r="F34" s="53" t="s">
+      <c r="F34" s="67" t="s">
         <v>31</v>
       </c>
-      <c r="G34" s="53"/>
-      <c r="H34" s="52" t="s">
+      <c r="G34" s="67"/>
+      <c r="H34" s="66" t="s">
         <v>32</v>
       </c>
-      <c r="I34" s="52"/>
-      <c r="J34" s="52"/>
-      <c r="K34" s="53" t="s">
+      <c r="I34" s="66"/>
+      <c r="J34" s="66"/>
+      <c r="K34" s="67" t="s">
         <v>33</v>
       </c>
-      <c r="L34" s="53"/>
-      <c r="M34" s="52" t="s">
+      <c r="L34" s="67"/>
+      <c r="M34" s="66" t="s">
         <v>2</v>
       </c>
-      <c r="N34" s="52"/>
-      <c r="O34" s="52"/>
+      <c r="N34" s="66"/>
+      <c r="O34" s="66"/>
     </row>
     <row r="35" spans="1:15" s="4" customFormat="1" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A35" s="52"/>
-      <c r="B35" s="52"/>
-      <c r="C35" s="53"/>
-      <c r="D35" s="53"/>
-      <c r="E35" s="53"/>
+      <c r="A35" s="66"/>
+      <c r="B35" s="66"/>
+      <c r="C35" s="67"/>
+      <c r="D35" s="67"/>
+      <c r="E35" s="67"/>
       <c r="F35" s="20" t="s">
         <v>21</v>
       </c>
@@ -2408,1179 +2409,1179 @@
         <v>46</v>
       </c>
     </row>
-    <row r="36" spans="1:15" ht="71.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:15" ht="135.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="23"/>
       <c r="B36" s="23"/>
       <c r="C36" s="24"/>
       <c r="D36" s="25"/>
       <c r="E36" s="26"/>
-      <c r="F36" s="30"/>
+      <c r="F36" s="40"/>
       <c r="G36" s="27"/>
       <c r="H36" s="21" t="str">
         <f t="shared" ref="H36:H41" si="0">IF(E36="Relacionada",IF(F36="Traslape Total","-",DATEDIF(C36,D36,"Y")),"-")</f>
         <v>-</v>
       </c>
       <c r="I36" s="21" t="str">
-        <f>IF(E220="Relacionada",IF(F36="Traslape Total","-",DATEDIF(C36,D36,"YM")),"-")</f>
+        <f t="shared" ref="I36:I66" si="1">IF(E220="Relacionada",IF(F36="Traslape Total","-",DATEDIF(C36,D36,"YM")),"-")</f>
         <v>-</v>
       </c>
       <c r="J36" s="21" t="str">
-        <f t="shared" ref="J36:J41" si="1">IF(E36="Relacionada",IF(F36="Traslape Total","-",DATEDIF(C36,D36,"Md")),"-")</f>
-        <v>-</v>
-      </c>
-      <c r="K36" s="28"/>
+        <f t="shared" ref="J36:J41" si="2">IF(E36="Relacionada",IF(F36="Traslape Total","-",DATEDIF(C36,D36,"Md")),"-")</f>
+        <v>-</v>
+      </c>
+      <c r="K36" s="41"/>
       <c r="L36" s="28"/>
       <c r="M36" s="29">
-        <f t="shared" ref="M36:M41" si="2">IF(K36="Traslape Total","-",DATEDIF(C36,D36,"Y"))</f>
+        <f t="shared" ref="M36:M41" si="3">IF(K36="Traslape Total","-",DATEDIF(C36,D36,"Y"))</f>
         <v>0</v>
       </c>
       <c r="N36" s="29">
-        <f t="shared" ref="N36:N41" si="3">IF(K36="Traslape Total","-",DATEDIF($C36,$D36,"YM"))</f>
+        <f t="shared" ref="N36:N41" si="4">IF(K36="Traslape Total","-",DATEDIF($C36,$D36,"YM"))</f>
         <v>0</v>
       </c>
       <c r="O36" s="29">
-        <f t="shared" ref="O36:O41" si="4">IF(K36="Traslape Total","-",DATEDIF($C36,$D36,"MD"))</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37" spans="1:15" ht="77.099999999999994" customHeight="1" x14ac:dyDescent="0.2">
+        <f t="shared" ref="O36:O41" si="5">IF(K36="Traslape Total","-",DATEDIF($C36,$D36,"MD"))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:15" ht="135.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="23"/>
       <c r="B37" s="23"/>
       <c r="C37" s="24"/>
       <c r="D37" s="25"/>
       <c r="E37" s="26"/>
-      <c r="F37" s="30"/>
+      <c r="F37" s="40"/>
       <c r="G37" s="27"/>
       <c r="H37" s="21" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
       <c r="I37" s="21" t="str">
-        <f>IF(E221="Relacionada",IF(F37="Traslape Total","-",DATEDIF(C37,D37,"YM")),"-")</f>
+        <f t="shared" si="1"/>
         <v>-</v>
       </c>
       <c r="J37" s="21" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-      <c r="K37" s="28"/>
+        <f t="shared" si="2"/>
+        <v>-</v>
+      </c>
+      <c r="K37" s="41"/>
       <c r="L37" s="28"/>
       <c r="M37" s="29">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="N37" s="29">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="O37" s="29">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="38" spans="1:15" ht="77.099999999999994" customHeight="1" x14ac:dyDescent="0.2">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:15" ht="135.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="23"/>
       <c r="B38" s="23"/>
       <c r="C38" s="24"/>
       <c r="D38" s="25"/>
       <c r="E38" s="26"/>
-      <c r="F38" s="30"/>
+      <c r="F38" s="40"/>
       <c r="G38" s="27"/>
       <c r="H38" s="21" t="str">
-        <f t="shared" ref="H38" si="5">IF(E38="Relacionada",IF(F38="Traslape Total","-",DATEDIF(C38,D38,"Y")),"-")</f>
+        <f t="shared" ref="H38" si="6">IF(E38="Relacionada",IF(F38="Traslape Total","-",DATEDIF(C38,D38,"Y")),"-")</f>
         <v>-</v>
       </c>
       <c r="I38" s="21" t="str">
-        <f>IF(E222="Relacionada",IF(F38="Traslape Total","-",DATEDIF(C38,D38,"YM")),"-")</f>
+        <f t="shared" si="1"/>
         <v>-</v>
       </c>
       <c r="J38" s="21" t="str">
-        <f t="shared" ref="J38" si="6">IF(E38="Relacionada",IF(F38="Traslape Total","-",DATEDIF(C38,D38,"Md")),"-")</f>
-        <v>-</v>
-      </c>
-      <c r="K38" s="28"/>
+        <f t="shared" ref="J38" si="7">IF(E38="Relacionada",IF(F38="Traslape Total","-",DATEDIF(C38,D38,"Md")),"-")</f>
+        <v>-</v>
+      </c>
+      <c r="K38" s="41"/>
       <c r="L38" s="28"/>
       <c r="M38" s="29">
-        <f t="shared" ref="M38" si="7">IF(K38="Traslape Total","-",DATEDIF(C38,D38,"Y"))</f>
+        <f t="shared" ref="M38" si="8">IF(K38="Traslape Total","-",DATEDIF(C38,D38,"Y"))</f>
         <v>0</v>
       </c>
       <c r="N38" s="29">
-        <f t="shared" ref="N38" si="8">IF(K38="Traslape Total","-",DATEDIF($C38,$D38,"YM"))</f>
+        <f t="shared" ref="N38" si="9">IF(K38="Traslape Total","-",DATEDIF($C38,$D38,"YM"))</f>
         <v>0</v>
       </c>
       <c r="O38" s="29">
-        <f t="shared" ref="O38" si="9">IF(K38="Traslape Total","-",DATEDIF($C38,$D38,"MD"))</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="39" spans="1:15" ht="77.099999999999994" customHeight="1" x14ac:dyDescent="0.2">
+        <f t="shared" ref="O38" si="10">IF(K38="Traslape Total","-",DATEDIF($C38,$D38,"MD"))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:15" ht="135.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="23"/>
       <c r="B39" s="23"/>
       <c r="C39" s="24"/>
       <c r="D39" s="25"/>
       <c r="E39" s="26"/>
-      <c r="F39" s="30"/>
+      <c r="F39" s="40"/>
       <c r="G39" s="27"/>
       <c r="H39" s="21" t="str">
-        <f t="shared" ref="H39:H40" si="10">IF(E39="Relacionada",IF(F39="Traslape Total","-",DATEDIF(C39,D39,"Y")),"-")</f>
+        <f t="shared" ref="H39:H40" si="11">IF(E39="Relacionada",IF(F39="Traslape Total","-",DATEDIF(C39,D39,"Y")),"-")</f>
         <v>-</v>
       </c>
       <c r="I39" s="21" t="str">
-        <f>IF(E223="Relacionada",IF(F39="Traslape Total","-",DATEDIF(C39,D39,"YM")),"-")</f>
+        <f t="shared" si="1"/>
         <v>-</v>
       </c>
       <c r="J39" s="21" t="str">
-        <f t="shared" ref="J39:J40" si="11">IF(E39="Relacionada",IF(F39="Traslape Total","-",DATEDIF(C39,D39,"Md")),"-")</f>
-        <v>-</v>
-      </c>
-      <c r="K39" s="28"/>
+        <f t="shared" ref="J39:J40" si="12">IF(E39="Relacionada",IF(F39="Traslape Total","-",DATEDIF(C39,D39,"Md")),"-")</f>
+        <v>-</v>
+      </c>
+      <c r="K39" s="41"/>
       <c r="L39" s="28"/>
       <c r="M39" s="29">
-        <f t="shared" ref="M39:M40" si="12">IF(K39="Traslape Total","-",DATEDIF(C39,D39,"Y"))</f>
+        <f t="shared" ref="M39:M40" si="13">IF(K39="Traslape Total","-",DATEDIF(C39,D39,"Y"))</f>
         <v>0</v>
       </c>
       <c r="N39" s="29">
-        <f t="shared" ref="N39:N40" si="13">IF(K39="Traslape Total","-",DATEDIF($C39,$D39,"YM"))</f>
+        <f t="shared" ref="N39:N40" si="14">IF(K39="Traslape Total","-",DATEDIF($C39,$D39,"YM"))</f>
         <v>0</v>
       </c>
       <c r="O39" s="29">
-        <f t="shared" ref="O39:O40" si="14">IF(K39="Traslape Total","-",DATEDIF($C39,$D39,"MD"))</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="40" spans="1:15" ht="81.75" customHeight="1" x14ac:dyDescent="0.2">
+        <f t="shared" ref="O39:O40" si="15">IF(K39="Traslape Total","-",DATEDIF($C39,$D39,"MD"))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:15" ht="135.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="23"/>
       <c r="B40" s="23"/>
       <c r="C40" s="24"/>
       <c r="D40" s="25"/>
       <c r="E40" s="26"/>
-      <c r="F40" s="30"/>
+      <c r="F40" s="40"/>
       <c r="G40" s="27"/>
       <c r="H40" s="21" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>-</v>
       </c>
       <c r="I40" s="21" t="str">
-        <f>IF(E224="Relacionada",IF(F40="Traslape Total","-",DATEDIF(C40,D40,"YM")),"-")</f>
+        <f t="shared" si="1"/>
         <v>-</v>
       </c>
       <c r="J40" s="21" t="str">
-        <f t="shared" si="11"/>
-        <v>-</v>
-      </c>
-      <c r="K40" s="28"/>
+        <f t="shared" si="12"/>
+        <v>-</v>
+      </c>
+      <c r="K40" s="41"/>
       <c r="L40" s="28"/>
       <c r="M40" s="29">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="N40" s="29">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>0</v>
       </c>
       <c r="O40" s="29">
-        <f t="shared" si="14"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="41" spans="1:15" ht="77.099999999999994" customHeight="1" x14ac:dyDescent="0.2">
+        <f t="shared" si="15"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:15" ht="135.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="23"/>
       <c r="B41" s="23"/>
       <c r="C41" s="24"/>
       <c r="D41" s="25"/>
       <c r="E41" s="26"/>
-      <c r="F41" s="30"/>
+      <c r="F41" s="40"/>
       <c r="G41" s="27"/>
       <c r="H41" s="21" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
       <c r="I41" s="21" t="str">
-        <f>IF(E225="Relacionada",IF(F41="Traslape Total","-",DATEDIF(C41,D41,"YM")),"-")</f>
+        <f t="shared" si="1"/>
         <v>-</v>
       </c>
       <c r="J41" s="21" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-      <c r="K41" s="28"/>
+        <f t="shared" si="2"/>
+        <v>-</v>
+      </c>
+      <c r="K41" s="41"/>
       <c r="L41" s="28"/>
       <c r="M41" s="29">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="N41" s="29">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="O41" s="29">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="42" spans="1:15" ht="77.099999999999994" customHeight="1" x14ac:dyDescent="0.2">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="1:15" ht="135.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="23"/>
       <c r="B42" s="23"/>
       <c r="C42" s="24"/>
       <c r="D42" s="25"/>
       <c r="E42" s="26"/>
-      <c r="F42" s="30"/>
+      <c r="F42" s="40"/>
       <c r="G42" s="27"/>
       <c r="H42" s="21" t="str">
-        <f t="shared" ref="H42:H66" si="15">IF(E42="Relacionada",IF(F42="Traslape Total","-",DATEDIF(C42,D42,"Y")),"-")</f>
+        <f t="shared" ref="H42:H66" si="16">IF(E42="Relacionada",IF(F42="Traslape Total","-",DATEDIF(C42,D42,"Y")),"-")</f>
         <v>-</v>
       </c>
       <c r="I42" s="21" t="str">
-        <f>IF(E226="Relacionada",IF(F42="Traslape Total","-",DATEDIF(C42,D42,"YM")),"-")</f>
+        <f t="shared" si="1"/>
         <v>-</v>
       </c>
       <c r="J42" s="21" t="str">
-        <f t="shared" ref="J42:J66" si="16">IF(E42="Relacionada",IF(F42="Traslape Total","-",DATEDIF(C42,D42,"Md")),"-")</f>
-        <v>-</v>
-      </c>
-      <c r="K42" s="28"/>
+        <f t="shared" ref="J42:J66" si="17">IF(E42="Relacionada",IF(F42="Traslape Total","-",DATEDIF(C42,D42,"Md")),"-")</f>
+        <v>-</v>
+      </c>
+      <c r="K42" s="41"/>
       <c r="L42" s="28"/>
       <c r="M42" s="29">
-        <f t="shared" ref="M42:M66" si="17">IF(K42="Traslape Total","-",DATEDIF(C42,D42,"Y"))</f>
+        <f t="shared" ref="M42:M66" si="18">IF(K42="Traslape Total","-",DATEDIF(C42,D42,"Y"))</f>
         <v>0</v>
       </c>
       <c r="N42" s="29">
-        <f t="shared" ref="N42:N66" si="18">IF(K42="Traslape Total","-",DATEDIF($C42,$D42,"YM"))</f>
+        <f t="shared" ref="N42:N66" si="19">IF(K42="Traslape Total","-",DATEDIF($C42,$D42,"YM"))</f>
         <v>0</v>
       </c>
       <c r="O42" s="29">
-        <f t="shared" ref="O42:O66" si="19">IF(K42="Traslape Total","-",DATEDIF($C42,$D42,"MD"))</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="43" spans="1:15" ht="77.099999999999994" customHeight="1" x14ac:dyDescent="0.2">
+        <f t="shared" ref="O42:O66" si="20">IF(K42="Traslape Total","-",DATEDIF($C42,$D42,"MD"))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:15" ht="135.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="23"/>
       <c r="B43" s="23"/>
       <c r="C43" s="24"/>
       <c r="D43" s="25"/>
       <c r="E43" s="26"/>
-      <c r="F43" s="30"/>
+      <c r="F43" s="40"/>
       <c r="G43" s="27"/>
       <c r="H43" s="21" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>-</v>
       </c>
       <c r="I43" s="21" t="str">
-        <f>IF(E227="Relacionada",IF(F43="Traslape Total","-",DATEDIF(C43,D43,"YM")),"-")</f>
+        <f t="shared" si="1"/>
         <v>-</v>
       </c>
       <c r="J43" s="21" t="str">
-        <f t="shared" si="16"/>
-        <v>-</v>
-      </c>
-      <c r="K43" s="28"/>
+        <f t="shared" si="17"/>
+        <v>-</v>
+      </c>
+      <c r="K43" s="41"/>
       <c r="L43" s="28"/>
       <c r="M43" s="29">
-        <f t="shared" si="17"/>
+        <f t="shared" si="18"/>
         <v>0</v>
       </c>
       <c r="N43" s="29">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>0</v>
       </c>
       <c r="O43" s="29">
-        <f t="shared" si="19"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="44" spans="1:15" ht="77.099999999999994" customHeight="1" x14ac:dyDescent="0.2">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" spans="1:15" ht="135.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="23"/>
       <c r="B44" s="23"/>
       <c r="C44" s="24"/>
       <c r="D44" s="25"/>
       <c r="E44" s="26"/>
-      <c r="F44" s="30"/>
+      <c r="F44" s="40"/>
       <c r="G44" s="27"/>
       <c r="H44" s="21" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>-</v>
       </c>
       <c r="I44" s="21" t="str">
-        <f>IF(E228="Relacionada",IF(F44="Traslape Total","-",DATEDIF(C44,D44,"YM")),"-")</f>
+        <f t="shared" si="1"/>
         <v>-</v>
       </c>
       <c r="J44" s="21" t="str">
-        <f t="shared" si="16"/>
-        <v>-</v>
-      </c>
-      <c r="K44" s="28"/>
+        <f t="shared" si="17"/>
+        <v>-</v>
+      </c>
+      <c r="K44" s="41"/>
       <c r="L44" s="28"/>
       <c r="M44" s="29">
-        <f t="shared" si="17"/>
+        <f t="shared" si="18"/>
         <v>0</v>
       </c>
       <c r="N44" s="29">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>0</v>
       </c>
       <c r="O44" s="29">
-        <f t="shared" si="19"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="45" spans="1:15" ht="77.099999999999994" customHeight="1" x14ac:dyDescent="0.2">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="1:15" ht="135.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="23"/>
       <c r="B45" s="23"/>
       <c r="C45" s="24"/>
       <c r="D45" s="25"/>
       <c r="E45" s="26"/>
-      <c r="F45" s="30"/>
+      <c r="F45" s="40"/>
       <c r="G45" s="27"/>
       <c r="H45" s="21" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>-</v>
       </c>
       <c r="I45" s="21" t="str">
-        <f>IF(E229="Relacionada",IF(F45="Traslape Total","-",DATEDIF(C45,D45,"YM")),"-")</f>
+        <f t="shared" si="1"/>
         <v>-</v>
       </c>
       <c r="J45" s="21" t="str">
-        <f t="shared" si="16"/>
-        <v>-</v>
-      </c>
-      <c r="K45" s="28"/>
+        <f t="shared" si="17"/>
+        <v>-</v>
+      </c>
+      <c r="K45" s="41"/>
       <c r="L45" s="28"/>
       <c r="M45" s="29">
-        <f t="shared" si="17"/>
+        <f t="shared" si="18"/>
         <v>0</v>
       </c>
       <c r="N45" s="29">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>0</v>
       </c>
       <c r="O45" s="29">
-        <f t="shared" si="19"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="46" spans="1:15" ht="77.099999999999994" customHeight="1" x14ac:dyDescent="0.2">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="1:15" ht="135.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="23"/>
       <c r="B46" s="23"/>
       <c r="C46" s="24"/>
       <c r="D46" s="25"/>
       <c r="E46" s="26"/>
-      <c r="F46" s="30"/>
+      <c r="F46" s="40"/>
       <c r="G46" s="27"/>
       <c r="H46" s="21" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>-</v>
       </c>
       <c r="I46" s="21" t="str">
-        <f>IF(E230="Relacionada",IF(F46="Traslape Total","-",DATEDIF(C46,D46,"YM")),"-")</f>
+        <f t="shared" si="1"/>
         <v>-</v>
       </c>
       <c r="J46" s="21" t="str">
-        <f t="shared" si="16"/>
-        <v>-</v>
-      </c>
-      <c r="K46" s="28"/>
+        <f t="shared" si="17"/>
+        <v>-</v>
+      </c>
+      <c r="K46" s="41"/>
       <c r="L46" s="28"/>
       <c r="M46" s="29">
-        <f t="shared" si="17"/>
+        <f t="shared" si="18"/>
         <v>0</v>
       </c>
       <c r="N46" s="29">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>0</v>
       </c>
       <c r="O46" s="29">
-        <f t="shared" si="19"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="47" spans="1:15" ht="77.099999999999994" customHeight="1" x14ac:dyDescent="0.2">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="1:15" ht="135.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="23"/>
       <c r="B47" s="23"/>
       <c r="C47" s="24"/>
       <c r="D47" s="25"/>
       <c r="E47" s="26"/>
-      <c r="F47" s="30"/>
+      <c r="F47" s="40"/>
       <c r="G47" s="27"/>
       <c r="H47" s="21" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>-</v>
       </c>
       <c r="I47" s="21" t="str">
-        <f>IF(E231="Relacionada",IF(F47="Traslape Total","-",DATEDIF(C47,D47,"YM")),"-")</f>
+        <f t="shared" si="1"/>
         <v>-</v>
       </c>
       <c r="J47" s="21" t="str">
-        <f t="shared" si="16"/>
-        <v>-</v>
-      </c>
-      <c r="K47" s="28"/>
+        <f t="shared" si="17"/>
+        <v>-</v>
+      </c>
+      <c r="K47" s="41"/>
       <c r="L47" s="28"/>
       <c r="M47" s="29">
-        <f t="shared" si="17"/>
+        <f t="shared" si="18"/>
         <v>0</v>
       </c>
       <c r="N47" s="29">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>0</v>
       </c>
       <c r="O47" s="29">
-        <f t="shared" si="19"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="48" spans="1:15" ht="77.099999999999994" customHeight="1" x14ac:dyDescent="0.2">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" spans="1:15" ht="135.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="23"/>
       <c r="B48" s="23"/>
       <c r="C48" s="24"/>
       <c r="D48" s="25"/>
       <c r="E48" s="26"/>
-      <c r="F48" s="30"/>
+      <c r="F48" s="40"/>
       <c r="G48" s="27"/>
       <c r="H48" s="21" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>-</v>
       </c>
       <c r="I48" s="21" t="str">
-        <f>IF(E232="Relacionada",IF(F48="Traslape Total","-",DATEDIF(C48,D48,"YM")),"-")</f>
+        <f t="shared" si="1"/>
         <v>-</v>
       </c>
       <c r="J48" s="21" t="str">
-        <f t="shared" si="16"/>
-        <v>-</v>
-      </c>
-      <c r="K48" s="28"/>
+        <f t="shared" si="17"/>
+        <v>-</v>
+      </c>
+      <c r="K48" s="41"/>
       <c r="L48" s="28"/>
       <c r="M48" s="29">
-        <f t="shared" si="17"/>
+        <f t="shared" si="18"/>
         <v>0</v>
       </c>
       <c r="N48" s="29">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>0</v>
       </c>
       <c r="O48" s="29">
-        <f t="shared" si="19"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="49" spans="1:15" ht="77.099999999999994" customHeight="1" x14ac:dyDescent="0.2">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" spans="1:15" ht="135.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="23"/>
       <c r="B49" s="23"/>
       <c r="C49" s="24"/>
       <c r="D49" s="25"/>
       <c r="E49" s="26"/>
-      <c r="F49" s="30"/>
+      <c r="F49" s="40"/>
       <c r="G49" s="27"/>
       <c r="H49" s="21" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>-</v>
       </c>
       <c r="I49" s="21" t="str">
-        <f>IF(E233="Relacionada",IF(F49="Traslape Total","-",DATEDIF(C49,D49,"YM")),"-")</f>
+        <f t="shared" si="1"/>
         <v>-</v>
       </c>
       <c r="J49" s="21" t="str">
-        <f t="shared" si="16"/>
-        <v>-</v>
-      </c>
-      <c r="K49" s="28"/>
+        <f t="shared" si="17"/>
+        <v>-</v>
+      </c>
+      <c r="K49" s="41"/>
       <c r="L49" s="28"/>
       <c r="M49" s="29">
-        <f t="shared" si="17"/>
+        <f t="shared" si="18"/>
         <v>0</v>
       </c>
       <c r="N49" s="29">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>0</v>
       </c>
       <c r="O49" s="29">
-        <f t="shared" si="19"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="50" spans="1:15" ht="77.099999999999994" customHeight="1" x14ac:dyDescent="0.2">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="1:15" ht="135.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="23"/>
       <c r="B50" s="23"/>
       <c r="C50" s="24"/>
       <c r="D50" s="25"/>
       <c r="E50" s="26"/>
-      <c r="F50" s="30"/>
+      <c r="F50" s="40"/>
       <c r="G50" s="27"/>
       <c r="H50" s="21" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>-</v>
       </c>
       <c r="I50" s="21" t="str">
-        <f>IF(E234="Relacionada",IF(F50="Traslape Total","-",DATEDIF(C50,D50,"YM")),"-")</f>
+        <f t="shared" si="1"/>
         <v>-</v>
       </c>
       <c r="J50" s="21" t="str">
-        <f t="shared" si="16"/>
-        <v>-</v>
-      </c>
-      <c r="K50" s="28"/>
+        <f t="shared" si="17"/>
+        <v>-</v>
+      </c>
+      <c r="K50" s="41"/>
       <c r="L50" s="28"/>
       <c r="M50" s="29">
-        <f t="shared" si="17"/>
+        <f t="shared" si="18"/>
         <v>0</v>
       </c>
       <c r="N50" s="29">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>0</v>
       </c>
       <c r="O50" s="29">
-        <f t="shared" si="19"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="51" spans="1:15" ht="77.099999999999994" customHeight="1" x14ac:dyDescent="0.2">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="1:15" ht="135.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="23"/>
       <c r="B51" s="23"/>
       <c r="C51" s="24"/>
       <c r="D51" s="25"/>
       <c r="E51" s="26"/>
-      <c r="F51" s="30"/>
+      <c r="F51" s="40"/>
       <c r="G51" s="27"/>
       <c r="H51" s="21" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>-</v>
       </c>
       <c r="I51" s="21" t="str">
-        <f>IF(E235="Relacionada",IF(F51="Traslape Total","-",DATEDIF(C51,D51,"YM")),"-")</f>
+        <f t="shared" si="1"/>
         <v>-</v>
       </c>
       <c r="J51" s="21" t="str">
-        <f t="shared" si="16"/>
-        <v>-</v>
-      </c>
-      <c r="K51" s="28"/>
+        <f t="shared" si="17"/>
+        <v>-</v>
+      </c>
+      <c r="K51" s="41"/>
       <c r="L51" s="28"/>
       <c r="M51" s="29">
-        <f t="shared" si="17"/>
+        <f t="shared" si="18"/>
         <v>0</v>
       </c>
       <c r="N51" s="29">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>0</v>
       </c>
       <c r="O51" s="29">
-        <f t="shared" si="19"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="52" spans="1:15" ht="77.099999999999994" customHeight="1" x14ac:dyDescent="0.2">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:15" ht="135.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="23"/>
       <c r="B52" s="23"/>
       <c r="C52" s="24"/>
       <c r="D52" s="25"/>
       <c r="E52" s="26"/>
-      <c r="F52" s="30"/>
+      <c r="F52" s="40"/>
       <c r="G52" s="27"/>
       <c r="H52" s="21" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>-</v>
       </c>
       <c r="I52" s="21" t="str">
-        <f>IF(E236="Relacionada",IF(F52="Traslape Total","-",DATEDIF(C52,D52,"YM")),"-")</f>
+        <f t="shared" si="1"/>
         <v>-</v>
       </c>
       <c r="J52" s="21" t="str">
-        <f t="shared" si="16"/>
-        <v>-</v>
-      </c>
-      <c r="K52" s="28"/>
+        <f t="shared" si="17"/>
+        <v>-</v>
+      </c>
+      <c r="K52" s="41"/>
       <c r="L52" s="28"/>
       <c r="M52" s="29">
-        <f t="shared" si="17"/>
+        <f t="shared" si="18"/>
         <v>0</v>
       </c>
       <c r="N52" s="29">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>0</v>
       </c>
       <c r="O52" s="29">
-        <f t="shared" si="19"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="53" spans="1:15" ht="77.099999999999994" customHeight="1" x14ac:dyDescent="0.2">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" spans="1:15" ht="135.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="23"/>
       <c r="B53" s="23"/>
       <c r="C53" s="24"/>
       <c r="D53" s="25"/>
       <c r="E53" s="26"/>
-      <c r="F53" s="30"/>
+      <c r="F53" s="40"/>
       <c r="G53" s="27"/>
       <c r="H53" s="21" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>-</v>
       </c>
       <c r="I53" s="21" t="str">
-        <f>IF(E237="Relacionada",IF(F53="Traslape Total","-",DATEDIF(C53,D53,"YM")),"-")</f>
+        <f t="shared" si="1"/>
         <v>-</v>
       </c>
       <c r="J53" s="21" t="str">
-        <f t="shared" si="16"/>
-        <v>-</v>
-      </c>
-      <c r="K53" s="28"/>
+        <f t="shared" si="17"/>
+        <v>-</v>
+      </c>
+      <c r="K53" s="41"/>
       <c r="L53" s="28"/>
       <c r="M53" s="29">
-        <f t="shared" si="17"/>
+        <f t="shared" si="18"/>
         <v>0</v>
       </c>
       <c r="N53" s="29">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>0</v>
       </c>
       <c r="O53" s="29">
-        <f t="shared" si="19"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="54" spans="1:15" ht="77.099999999999994" customHeight="1" x14ac:dyDescent="0.2">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54" spans="1:15" ht="135.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" s="23"/>
       <c r="B54" s="23"/>
       <c r="C54" s="24"/>
       <c r="D54" s="25"/>
       <c r="E54" s="26"/>
-      <c r="F54" s="30"/>
+      <c r="F54" s="40"/>
       <c r="G54" s="27"/>
       <c r="H54" s="21" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>-</v>
       </c>
       <c r="I54" s="21" t="str">
-        <f>IF(E238="Relacionada",IF(F54="Traslape Total","-",DATEDIF(C54,D54,"YM")),"-")</f>
+        <f t="shared" si="1"/>
         <v>-</v>
       </c>
       <c r="J54" s="21" t="str">
-        <f t="shared" si="16"/>
-        <v>-</v>
-      </c>
-      <c r="K54" s="28"/>
+        <f t="shared" si="17"/>
+        <v>-</v>
+      </c>
+      <c r="K54" s="41"/>
       <c r="L54" s="28"/>
       <c r="M54" s="29">
-        <f t="shared" si="17"/>
+        <f t="shared" si="18"/>
         <v>0</v>
       </c>
       <c r="N54" s="29">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>0</v>
       </c>
       <c r="O54" s="29">
-        <f t="shared" si="19"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="55" spans="1:15" ht="77.099999999999994" customHeight="1" x14ac:dyDescent="0.2">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55" spans="1:15" ht="135.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="23"/>
       <c r="B55" s="23"/>
       <c r="C55" s="24"/>
       <c r="D55" s="25"/>
       <c r="E55" s="26"/>
-      <c r="F55" s="30"/>
+      <c r="F55" s="40"/>
       <c r="G55" s="27"/>
       <c r="H55" s="21" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>-</v>
       </c>
       <c r="I55" s="21" t="str">
-        <f>IF(E239="Relacionada",IF(F55="Traslape Total","-",DATEDIF(C55,D55,"YM")),"-")</f>
+        <f t="shared" si="1"/>
         <v>-</v>
       </c>
       <c r="J55" s="21" t="str">
-        <f t="shared" si="16"/>
-        <v>-</v>
-      </c>
-      <c r="K55" s="28"/>
+        <f t="shared" si="17"/>
+        <v>-</v>
+      </c>
+      <c r="K55" s="41"/>
       <c r="L55" s="28"/>
       <c r="M55" s="29">
-        <f t="shared" si="17"/>
+        <f t="shared" si="18"/>
         <v>0</v>
       </c>
       <c r="N55" s="29">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>0</v>
       </c>
       <c r="O55" s="29">
-        <f t="shared" si="19"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="56" spans="1:15" ht="77.099999999999994" customHeight="1" x14ac:dyDescent="0.2">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" spans="1:15" ht="135.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56" s="23"/>
       <c r="B56" s="23"/>
       <c r="C56" s="24"/>
       <c r="D56" s="25"/>
       <c r="E56" s="26"/>
-      <c r="F56" s="30"/>
+      <c r="F56" s="40"/>
       <c r="G56" s="27"/>
       <c r="H56" s="21" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>-</v>
       </c>
       <c r="I56" s="21" t="str">
-        <f>IF(E240="Relacionada",IF(F56="Traslape Total","-",DATEDIF(C56,D56,"YM")),"-")</f>
+        <f t="shared" si="1"/>
         <v>-</v>
       </c>
       <c r="J56" s="21" t="str">
-        <f t="shared" si="16"/>
-        <v>-</v>
-      </c>
-      <c r="K56" s="28"/>
+        <f t="shared" si="17"/>
+        <v>-</v>
+      </c>
+      <c r="K56" s="41"/>
       <c r="L56" s="28"/>
       <c r="M56" s="29">
-        <f t="shared" si="17"/>
+        <f t="shared" si="18"/>
         <v>0</v>
       </c>
       <c r="N56" s="29">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>0</v>
       </c>
       <c r="O56" s="29">
-        <f t="shared" si="19"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="57" spans="1:15" ht="77.099999999999994" customHeight="1" x14ac:dyDescent="0.2">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" spans="1:15" ht="135.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" s="23"/>
       <c r="B57" s="23"/>
       <c r="C57" s="24"/>
       <c r="D57" s="25"/>
       <c r="E57" s="26"/>
-      <c r="F57" s="30"/>
+      <c r="F57" s="40"/>
       <c r="G57" s="27"/>
       <c r="H57" s="21" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>-</v>
       </c>
       <c r="I57" s="21" t="str">
-        <f>IF(E241="Relacionada",IF(F57="Traslape Total","-",DATEDIF(C57,D57,"YM")),"-")</f>
+        <f t="shared" si="1"/>
         <v>-</v>
       </c>
       <c r="J57" s="21" t="str">
-        <f t="shared" si="16"/>
-        <v>-</v>
-      </c>
-      <c r="K57" s="28"/>
+        <f t="shared" si="17"/>
+        <v>-</v>
+      </c>
+      <c r="K57" s="41"/>
       <c r="L57" s="28"/>
       <c r="M57" s="29">
-        <f t="shared" si="17"/>
+        <f t="shared" si="18"/>
         <v>0</v>
       </c>
       <c r="N57" s="29">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>0</v>
       </c>
       <c r="O57" s="29">
-        <f t="shared" si="19"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="58" spans="1:15" ht="77.099999999999994" customHeight="1" x14ac:dyDescent="0.2">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58" spans="1:15" ht="135.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="23"/>
       <c r="B58" s="23"/>
       <c r="C58" s="24"/>
       <c r="D58" s="25"/>
       <c r="E58" s="26"/>
-      <c r="F58" s="30"/>
+      <c r="F58" s="40"/>
       <c r="G58" s="27"/>
       <c r="H58" s="21" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>-</v>
       </c>
       <c r="I58" s="21" t="str">
-        <f>IF(E242="Relacionada",IF(F58="Traslape Total","-",DATEDIF(C58,D58,"YM")),"-")</f>
+        <f t="shared" si="1"/>
         <v>-</v>
       </c>
       <c r="J58" s="21" t="str">
-        <f t="shared" si="16"/>
-        <v>-</v>
-      </c>
-      <c r="K58" s="28"/>
+        <f t="shared" si="17"/>
+        <v>-</v>
+      </c>
+      <c r="K58" s="41"/>
       <c r="L58" s="28"/>
       <c r="M58" s="29">
-        <f t="shared" si="17"/>
+        <f t="shared" si="18"/>
         <v>0</v>
       </c>
       <c r="N58" s="29">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>0</v>
       </c>
       <c r="O58" s="29">
-        <f t="shared" si="19"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="59" spans="1:15" ht="77.099999999999994" customHeight="1" x14ac:dyDescent="0.2">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59" spans="1:15" ht="135.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" s="23"/>
       <c r="B59" s="23"/>
       <c r="C59" s="24"/>
       <c r="D59" s="25"/>
       <c r="E59" s="26"/>
-      <c r="F59" s="30"/>
+      <c r="F59" s="40"/>
       <c r="G59" s="27"/>
       <c r="H59" s="21" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>-</v>
       </c>
       <c r="I59" s="21" t="str">
-        <f>IF(E243="Relacionada",IF(F59="Traslape Total","-",DATEDIF(C59,D59,"YM")),"-")</f>
+        <f t="shared" si="1"/>
         <v>-</v>
       </c>
       <c r="J59" s="21" t="str">
-        <f t="shared" si="16"/>
-        <v>-</v>
-      </c>
-      <c r="K59" s="28"/>
+        <f t="shared" si="17"/>
+        <v>-</v>
+      </c>
+      <c r="K59" s="41"/>
       <c r="L59" s="28"/>
       <c r="M59" s="29">
-        <f t="shared" si="17"/>
+        <f t="shared" si="18"/>
         <v>0</v>
       </c>
       <c r="N59" s="29">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>0</v>
       </c>
       <c r="O59" s="29">
-        <f t="shared" si="19"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="60" spans="1:15" ht="77.099999999999994" customHeight="1" x14ac:dyDescent="0.2">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60" spans="1:15" ht="135.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" s="23"/>
       <c r="B60" s="23"/>
       <c r="C60" s="24"/>
       <c r="D60" s="25"/>
       <c r="E60" s="26"/>
-      <c r="F60" s="30"/>
+      <c r="F60" s="40"/>
       <c r="G60" s="27"/>
       <c r="H60" s="21" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>-</v>
       </c>
       <c r="I60" s="21" t="str">
-        <f>IF(E244="Relacionada",IF(F60="Traslape Total","-",DATEDIF(C60,D60,"YM")),"-")</f>
+        <f t="shared" si="1"/>
         <v>-</v>
       </c>
       <c r="J60" s="21" t="str">
-        <f t="shared" si="16"/>
-        <v>-</v>
-      </c>
-      <c r="K60" s="28"/>
+        <f t="shared" si="17"/>
+        <v>-</v>
+      </c>
+      <c r="K60" s="41"/>
       <c r="L60" s="28"/>
       <c r="M60" s="29">
-        <f t="shared" si="17"/>
+        <f t="shared" si="18"/>
         <v>0</v>
       </c>
       <c r="N60" s="29">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>0</v>
       </c>
       <c r="O60" s="29">
-        <f t="shared" si="19"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="61" spans="1:15" ht="77.099999999999994" customHeight="1" x14ac:dyDescent="0.2">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61" spans="1:15" ht="135.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A61" s="23"/>
       <c r="B61" s="23"/>
       <c r="C61" s="24"/>
       <c r="D61" s="25"/>
       <c r="E61" s="26"/>
-      <c r="F61" s="30"/>
+      <c r="F61" s="40"/>
       <c r="G61" s="27"/>
       <c r="H61" s="21" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>-</v>
       </c>
       <c r="I61" s="21" t="str">
-        <f>IF(E245="Relacionada",IF(F61="Traslape Total","-",DATEDIF(C61,D61,"YM")),"-")</f>
+        <f t="shared" si="1"/>
         <v>-</v>
       </c>
       <c r="J61" s="21" t="str">
-        <f t="shared" si="16"/>
-        <v>-</v>
-      </c>
-      <c r="K61" s="28"/>
+        <f t="shared" si="17"/>
+        <v>-</v>
+      </c>
+      <c r="K61" s="41"/>
       <c r="L61" s="28"/>
       <c r="M61" s="29">
-        <f t="shared" si="17"/>
+        <f t="shared" si="18"/>
         <v>0</v>
       </c>
       <c r="N61" s="29">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>0</v>
       </c>
       <c r="O61" s="29">
-        <f t="shared" si="19"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="62" spans="1:15" ht="77.099999999999994" customHeight="1" x14ac:dyDescent="0.2">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" spans="1:15" ht="135.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A62" s="23"/>
       <c r="B62" s="23"/>
       <c r="C62" s="24"/>
       <c r="D62" s="25"/>
       <c r="E62" s="26"/>
-      <c r="F62" s="30"/>
+      <c r="F62" s="40"/>
       <c r="G62" s="27"/>
       <c r="H62" s="21" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>-</v>
       </c>
       <c r="I62" s="21" t="str">
-        <f>IF(E246="Relacionada",IF(F62="Traslape Total","-",DATEDIF(C62,D62,"YM")),"-")</f>
+        <f t="shared" si="1"/>
         <v>-</v>
       </c>
       <c r="J62" s="21" t="str">
-        <f t="shared" si="16"/>
-        <v>-</v>
-      </c>
-      <c r="K62" s="28"/>
+        <f t="shared" si="17"/>
+        <v>-</v>
+      </c>
+      <c r="K62" s="41"/>
       <c r="L62" s="28"/>
       <c r="M62" s="29">
-        <f t="shared" si="17"/>
+        <f t="shared" si="18"/>
         <v>0</v>
       </c>
       <c r="N62" s="29">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>0</v>
       </c>
       <c r="O62" s="29">
-        <f t="shared" si="19"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="63" spans="1:15" ht="77.099999999999994" customHeight="1" x14ac:dyDescent="0.2">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" spans="1:15" ht="135.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A63" s="23"/>
       <c r="B63" s="23"/>
       <c r="C63" s="24"/>
       <c r="D63" s="25"/>
       <c r="E63" s="26"/>
-      <c r="F63" s="30"/>
+      <c r="F63" s="40"/>
       <c r="G63" s="27"/>
       <c r="H63" s="21" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>-</v>
       </c>
       <c r="I63" s="21" t="str">
-        <f>IF(E247="Relacionada",IF(F63="Traslape Total","-",DATEDIF(C63,D63,"YM")),"-")</f>
+        <f t="shared" si="1"/>
         <v>-</v>
       </c>
       <c r="J63" s="21" t="str">
-        <f t="shared" si="16"/>
-        <v>-</v>
-      </c>
-      <c r="K63" s="28"/>
+        <f t="shared" si="17"/>
+        <v>-</v>
+      </c>
+      <c r="K63" s="41"/>
       <c r="L63" s="28"/>
       <c r="M63" s="29">
-        <f t="shared" si="17"/>
+        <f t="shared" si="18"/>
         <v>0</v>
       </c>
       <c r="N63" s="29">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>0</v>
       </c>
       <c r="O63" s="29">
-        <f t="shared" si="19"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="64" spans="1:15" ht="77.099999999999994" customHeight="1" x14ac:dyDescent="0.2">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64" spans="1:15" ht="135.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A64" s="23"/>
       <c r="B64" s="23"/>
       <c r="C64" s="24"/>
       <c r="D64" s="25"/>
       <c r="E64" s="26"/>
-      <c r="F64" s="30"/>
+      <c r="F64" s="40"/>
       <c r="G64" s="27"/>
       <c r="H64" s="21" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>-</v>
       </c>
       <c r="I64" s="21" t="str">
-        <f>IF(E248="Relacionada",IF(F64="Traslape Total","-",DATEDIF(C64,D64,"YM")),"-")</f>
+        <f t="shared" si="1"/>
         <v>-</v>
       </c>
       <c r="J64" s="21" t="str">
-        <f t="shared" si="16"/>
-        <v>-</v>
-      </c>
-      <c r="K64" s="28"/>
+        <f t="shared" si="17"/>
+        <v>-</v>
+      </c>
+      <c r="K64" s="41"/>
       <c r="L64" s="28"/>
       <c r="M64" s="29">
-        <f t="shared" si="17"/>
+        <f t="shared" si="18"/>
         <v>0</v>
       </c>
       <c r="N64" s="29">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>0</v>
       </c>
       <c r="O64" s="29">
-        <f t="shared" si="19"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="65" spans="1:18" ht="77.099999999999994" customHeight="1" x14ac:dyDescent="0.2">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65" spans="1:18" ht="135.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A65" s="23"/>
       <c r="B65" s="23"/>
       <c r="C65" s="24"/>
       <c r="D65" s="25"/>
       <c r="E65" s="26"/>
-      <c r="F65" s="30"/>
+      <c r="F65" s="40"/>
       <c r="G65" s="27"/>
       <c r="H65" s="21" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>-</v>
       </c>
       <c r="I65" s="21" t="str">
-        <f>IF(E249="Relacionada",IF(F65="Traslape Total","-",DATEDIF(C65,D65,"YM")),"-")</f>
+        <f t="shared" si="1"/>
         <v>-</v>
       </c>
       <c r="J65" s="21" t="str">
-        <f t="shared" si="16"/>
-        <v>-</v>
-      </c>
-      <c r="K65" s="28"/>
+        <f t="shared" si="17"/>
+        <v>-</v>
+      </c>
+      <c r="K65" s="41"/>
       <c r="L65" s="28"/>
       <c r="M65" s="29">
-        <f t="shared" si="17"/>
+        <f t="shared" si="18"/>
         <v>0</v>
       </c>
       <c r="N65" s="29">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>0</v>
       </c>
       <c r="O65" s="29">
-        <f t="shared" si="19"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="66" spans="1:18" ht="77.099999999999994" customHeight="1" x14ac:dyDescent="0.2">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66" spans="1:18" ht="135.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A66" s="23"/>
       <c r="B66" s="23"/>
       <c r="C66" s="24"/>
       <c r="D66" s="25"/>
       <c r="E66" s="26"/>
-      <c r="F66" s="30"/>
+      <c r="F66" s="40"/>
       <c r="G66" s="27"/>
       <c r="H66" s="21" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>-</v>
       </c>
       <c r="I66" s="21" t="str">
-        <f>IF(E250="Relacionada",IF(F66="Traslape Total","-",DATEDIF(C66,D66,"YM")),"-")</f>
+        <f t="shared" si="1"/>
         <v>-</v>
       </c>
       <c r="J66" s="21" t="str">
-        <f t="shared" si="16"/>
-        <v>-</v>
-      </c>
-      <c r="K66" s="28"/>
+        <f t="shared" si="17"/>
+        <v>-</v>
+      </c>
+      <c r="K66" s="41"/>
       <c r="L66" s="28"/>
       <c r="M66" s="29">
-        <f t="shared" si="17"/>
+        <f t="shared" si="18"/>
         <v>0</v>
       </c>
       <c r="N66" s="29">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>0</v>
       </c>
       <c r="O66" s="29">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>0</v>
       </c>
     </row>
     <row r="67" spans="1:18" s="4" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A67" s="50" t="s">
+      <c r="A67" s="64" t="s">
         <v>2</v>
       </c>
-      <c r="B67" s="50"/>
-      <c r="C67" s="50"/>
-      <c r="D67" s="50"/>
-      <c r="E67" s="50"/>
-      <c r="F67" s="51" t="s">
+      <c r="B67" s="64"/>
+      <c r="C67" s="64"/>
+      <c r="D67" s="64"/>
+      <c r="E67" s="64"/>
+      <c r="F67" s="65" t="s">
         <v>35</v>
       </c>
-      <c r="G67" s="51"/>
-      <c r="H67" s="33">
+      <c r="G67" s="65"/>
+      <c r="H67" s="32">
         <f>SUM(H36:H66)</f>
         <v>0</v>
       </c>
-      <c r="I67" s="33">
+      <c r="I67" s="32">
         <f>SUM(I36:I66)</f>
         <v>0</v>
       </c>
-      <c r="J67" s="33">
+      <c r="J67" s="32">
         <f>SUM(J36:J66)</f>
         <v>0</v>
       </c>
-      <c r="K67" s="51" t="s">
+      <c r="K67" s="65" t="s">
         <v>36</v>
       </c>
-      <c r="L67" s="51"/>
-      <c r="M67" s="33">
+      <c r="L67" s="65"/>
+      <c r="M67" s="32">
         <f>SUM(M36:M66)</f>
         <v>0</v>
       </c>
-      <c r="N67" s="33">
+      <c r="N67" s="32">
         <f>SUM(N36:N66)</f>
         <v>0</v>
       </c>
-      <c r="O67" s="33">
+      <c r="O67" s="32">
         <f>SUM(O36:O66)</f>
         <v>0</v>
       </c>
     </row>
     <row r="68" spans="1:18" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A68" s="49" t="s">
+      <c r="A68" s="61" t="s">
         <v>3</v>
       </c>
-      <c r="B68" s="49"/>
-      <c r="C68" s="49"/>
-      <c r="D68" s="49"/>
-      <c r="E68" s="49"/>
-      <c r="F68" s="51"/>
-      <c r="G68" s="51"/>
-      <c r="H68" s="34">
+      <c r="B68" s="61"/>
+      <c r="C68" s="61"/>
+      <c r="D68" s="61"/>
+      <c r="E68" s="61"/>
+      <c r="F68" s="65"/>
+      <c r="G68" s="65"/>
+      <c r="H68" s="33">
         <f>+INT((SUM(I36:I66)+INT((SUM(J36:J66)/30)))/12)+H67</f>
         <v>0</v>
       </c>
-      <c r="I68" s="35">
+      <c r="I68" s="34">
         <f>(((SUM(I36:I66)+INT(SUM(J36:J66)/30))/12)-(INT((SUM(I36:I66)+INT((SUM(J36:J66)/30)))/12)))*12</f>
         <v>0</v>
       </c>
-      <c r="J68" s="36">
+      <c r="J68" s="35">
         <f>(SUM(J36:J66)/30-INT(SUM(J36:J66)/30))*30</f>
         <v>0</v>
       </c>
-      <c r="K68" s="51"/>
-      <c r="L68" s="51"/>
-      <c r="M68" s="34">
+      <c r="K68" s="65"/>
+      <c r="L68" s="65"/>
+      <c r="M68" s="33">
         <f>+INT((SUM(N36:N66)+INT((SUM(O36:O66)/30)))/12)+M67</f>
         <v>0</v>
       </c>
-      <c r="N68" s="35">
+      <c r="N68" s="34">
         <f>(((SUM(N36:N66)+INT(SUM(O36:O66)/30))/12)-(INT((SUM(N36:N66)+INT((SUM(O36:O66)/30)))/12)))*12</f>
         <v>0</v>
       </c>
-      <c r="O68" s="36">
+      <c r="O68" s="35">
         <f>(SUM(O36:O66)/30-INT(SUM(O36:O66)/30))*30</f>
         <v>0</v>
       </c>
     </row>
     <row r="69" spans="1:18" ht="47.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A69" s="31"/>
-      <c r="B69" s="32"/>
-      <c r="C69" s="32"/>
-      <c r="D69" s="32"/>
-      <c r="E69" s="32"/>
-      <c r="F69" s="32"/>
-      <c r="G69" s="32"/>
-      <c r="H69" s="32"/>
-      <c r="I69" s="32"/>
+      <c r="A69" s="30"/>
+      <c r="B69" s="31"/>
+      <c r="C69" s="31"/>
+      <c r="D69" s="31"/>
+      <c r="E69" s="31"/>
+      <c r="F69" s="31"/>
+      <c r="G69" s="31"/>
+      <c r="H69" s="31"/>
+      <c r="I69" s="31"/>
       <c r="J69" s="19"/>
       <c r="K69" s="19"/>
       <c r="L69" s="19"/>
@@ -3614,11 +3615,11 @@
       <c r="B71" s="19"/>
       <c r="C71" s="19"/>
       <c r="D71" s="19"/>
-      <c r="E71" s="46" t="s">
+      <c r="E71" s="58" t="s">
         <v>38</v>
       </c>
-      <c r="F71" s="46"/>
-      <c r="G71" s="46"/>
+      <c r="F71" s="58"/>
+      <c r="G71" s="58"/>
       <c r="H71" s="19"/>
       <c r="I71" s="19"/>
       <c r="J71" s="19"/>
@@ -3704,7 +3705,6 @@
     </row>
   </sheetData>
   <mergeCells count="146">
-    <mergeCell ref="N30:O30"/>
     <mergeCell ref="B29:D29"/>
     <mergeCell ref="E29:G29"/>
     <mergeCell ref="H29:K29"/>
@@ -3735,24 +3735,6 @@
     <mergeCell ref="H23:K23"/>
     <mergeCell ref="L23:M23"/>
     <mergeCell ref="N23:O23"/>
-    <mergeCell ref="B22:D22"/>
-    <mergeCell ref="E22:G22"/>
-    <mergeCell ref="H22:K22"/>
-    <mergeCell ref="L22:M22"/>
-    <mergeCell ref="N22:O22"/>
-    <mergeCell ref="N19:O19"/>
-    <mergeCell ref="B21:D21"/>
-    <mergeCell ref="E21:G21"/>
-    <mergeCell ref="H21:K21"/>
-    <mergeCell ref="L21:M21"/>
-    <mergeCell ref="N21:O21"/>
-    <mergeCell ref="N17:O17"/>
-    <mergeCell ref="B18:D18"/>
-    <mergeCell ref="E18:G18"/>
-    <mergeCell ref="H18:K18"/>
-    <mergeCell ref="L18:M18"/>
-    <mergeCell ref="N18:O18"/>
-    <mergeCell ref="N13:O13"/>
     <mergeCell ref="B16:D16"/>
     <mergeCell ref="E16:G16"/>
     <mergeCell ref="H16:K16"/>
@@ -3773,10 +3755,6 @@
     <mergeCell ref="A3:N3"/>
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="D1:O1"/>
-    <mergeCell ref="F34:G34"/>
-    <mergeCell ref="H34:J34"/>
-    <mergeCell ref="K34:L34"/>
-    <mergeCell ref="M34:O34"/>
     <mergeCell ref="A8:F8"/>
     <mergeCell ref="G8:O8"/>
     <mergeCell ref="A7:F7"/>
@@ -3787,30 +3765,37 @@
     <mergeCell ref="N5:O5"/>
     <mergeCell ref="F4:G4"/>
     <mergeCell ref="M4:O4"/>
-    <mergeCell ref="A67:E67"/>
-    <mergeCell ref="H5:I5"/>
-    <mergeCell ref="J5:K5"/>
-    <mergeCell ref="F67:G68"/>
-    <mergeCell ref="L30:M30"/>
-    <mergeCell ref="K67:L68"/>
-    <mergeCell ref="A34:A35"/>
-    <mergeCell ref="B34:B35"/>
-    <mergeCell ref="C34:C35"/>
-    <mergeCell ref="D34:D35"/>
-    <mergeCell ref="E34:E35"/>
-    <mergeCell ref="B15:D15"/>
-    <mergeCell ref="E15:G15"/>
-    <mergeCell ref="H15:K15"/>
-    <mergeCell ref="L15:M15"/>
-    <mergeCell ref="B13:D13"/>
-    <mergeCell ref="L31:M31"/>
-    <mergeCell ref="B31:D31"/>
-    <mergeCell ref="E11:G11"/>
-    <mergeCell ref="H11:K11"/>
-    <mergeCell ref="L11:M11"/>
-    <mergeCell ref="E13:G13"/>
-    <mergeCell ref="H13:K13"/>
-    <mergeCell ref="L13:M13"/>
+    <mergeCell ref="B24:D24"/>
+    <mergeCell ref="E20:G20"/>
+    <mergeCell ref="B18:D18"/>
+    <mergeCell ref="E18:G18"/>
+    <mergeCell ref="H18:K18"/>
+    <mergeCell ref="L18:M18"/>
+    <mergeCell ref="B22:D22"/>
+    <mergeCell ref="E22:G22"/>
+    <mergeCell ref="H22:K22"/>
+    <mergeCell ref="L22:M22"/>
+    <mergeCell ref="B21:D21"/>
+    <mergeCell ref="E21:G21"/>
+    <mergeCell ref="H21:K21"/>
+    <mergeCell ref="L21:M21"/>
+    <mergeCell ref="F34:G34"/>
+    <mergeCell ref="H34:J34"/>
+    <mergeCell ref="K34:L34"/>
+    <mergeCell ref="M34:O34"/>
+    <mergeCell ref="N17:O17"/>
+    <mergeCell ref="N18:O18"/>
+    <mergeCell ref="N13:O13"/>
+    <mergeCell ref="N22:O22"/>
+    <mergeCell ref="N19:O19"/>
+    <mergeCell ref="N21:O21"/>
+    <mergeCell ref="N30:O30"/>
+    <mergeCell ref="A33:O33"/>
+    <mergeCell ref="N31:O31"/>
+    <mergeCell ref="B30:D30"/>
+    <mergeCell ref="E30:G30"/>
+    <mergeCell ref="H30:K30"/>
+    <mergeCell ref="E32:G32"/>
     <mergeCell ref="B17:D17"/>
     <mergeCell ref="E17:G17"/>
     <mergeCell ref="H17:K17"/>
@@ -3818,9 +3803,6 @@
     <mergeCell ref="B19:D19"/>
     <mergeCell ref="E19:G19"/>
     <mergeCell ref="H19:K19"/>
-    <mergeCell ref="L19:M19"/>
-    <mergeCell ref="B24:D24"/>
-    <mergeCell ref="E20:G20"/>
     <mergeCell ref="E71:G71"/>
     <mergeCell ref="L5:M5"/>
     <mergeCell ref="B5:C5"/>
@@ -3834,14 +3816,21 @@
     <mergeCell ref="H20:K20"/>
     <mergeCell ref="E31:G31"/>
     <mergeCell ref="H31:K31"/>
-    <mergeCell ref="N11:O11"/>
-    <mergeCell ref="N12:O12"/>
-    <mergeCell ref="A33:O33"/>
-    <mergeCell ref="N31:O31"/>
-    <mergeCell ref="B30:D30"/>
-    <mergeCell ref="E30:G30"/>
-    <mergeCell ref="H30:K30"/>
-    <mergeCell ref="E32:G32"/>
+    <mergeCell ref="A67:E67"/>
+    <mergeCell ref="H5:I5"/>
+    <mergeCell ref="J5:K5"/>
+    <mergeCell ref="F67:G68"/>
+    <mergeCell ref="L30:M30"/>
+    <mergeCell ref="K67:L68"/>
+    <mergeCell ref="A34:A35"/>
+    <mergeCell ref="B34:B35"/>
+    <mergeCell ref="C34:C35"/>
+    <mergeCell ref="D34:D35"/>
+    <mergeCell ref="E34:E35"/>
+    <mergeCell ref="B13:D13"/>
+    <mergeCell ref="L31:M31"/>
+    <mergeCell ref="B31:D31"/>
+    <mergeCell ref="E11:G11"/>
     <mergeCell ref="H32:K32"/>
     <mergeCell ref="B32:D32"/>
     <mergeCell ref="N20:O20"/>
@@ -3850,15 +3839,27 @@
     <mergeCell ref="H24:K24"/>
     <mergeCell ref="L24:M24"/>
     <mergeCell ref="N24:O24"/>
+    <mergeCell ref="B15:D15"/>
+    <mergeCell ref="E15:G15"/>
+    <mergeCell ref="H15:K15"/>
+    <mergeCell ref="L15:M15"/>
+    <mergeCell ref="H11:K11"/>
+    <mergeCell ref="L11:M11"/>
+    <mergeCell ref="E13:G13"/>
+    <mergeCell ref="H13:K13"/>
+    <mergeCell ref="L13:M13"/>
+    <mergeCell ref="N11:O11"/>
+    <mergeCell ref="N12:O12"/>
+    <mergeCell ref="L19:M19"/>
   </mergeCells>
-  <dataValidations disablePrompts="1" count="1">
+  <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E36:E66" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Relacionada,Profesional,Laboral"</formula1>
     </dataValidation>
   </dataValidations>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.23622047244094491" right="0.23622047244094491" top="0.39370078740157483" bottom="1.3779527559055118" header="0.19685039370078741" footer="0.19685039370078741"/>
-  <pageSetup scale="49" orientation="portrait" horizontalDpi="4294967294" verticalDpi="4294967294" r:id="rId1"/>
+  <pageSetup scale="47" fitToHeight="0" orientation="portrait" horizontalDpi="4294967294" verticalDpi="4294967294" r:id="rId1"/>
   <headerFooter>
     <oddFooter>&amp;C&amp;"Arial,Negrita"&amp;16&amp;G
 CLASIFICACIÓN DE LA INFORMACIÓN: PÚBLICA CLASIFICADA

</xml_diff>